<commit_message>
[greenjobs] Test coverage 78% -> 99%: recorded scraper corpus, branch tests, dashboard DOM test, honest skips, mutation-checked assertions
Scraper: parse_salary repairs mojibake pound signs (found by the fixture).
test_build: main guard moved to end so panel-B tests run; two stale expectations corrected.

Co-Authored-By: Claude <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XyZXNeMjVmnqRyKctLtDmB
</commit_message>
<xml_diff>
--- a/deliverables/greenjobs_redesign_2026-09-22/tests_register_2026-09-28.xlsx
+++ b/deliverables/greenjobs_redesign_2026-09-22/tests_register_2026-09-28.xlsx
@@ -8,16 +8,18 @@
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Manual cases" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Automated Python" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Automated Node" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Not automatable" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Coverage" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Manual cases" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Automated Python" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Automated Node" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Not automatable" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Manual cases'!$A$1:$G$46</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Automated Python'!$A$1:$E$44</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Automated Node'!$A$1:$B$36</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Not automatable'!$A$1:$C$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Coverage'!$A$1:$D$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Manual cases'!$A$1:$G$46</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Automated Python'!$A$1:$E$69</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Automated Node'!$A$1:$B$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Not automatable'!$A$1:$C$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -446,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -487,7 +489,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>43 test functions, 319 checks, 0 failed</t>
+          <t>68 test functions across 3 files; 575 checks (test_build run incl. companions) + 126 gap checks + 87 scraper checks; 0 failed, 0 skipped</t>
         </is>
       </c>
     </row>
@@ -499,7 +501,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>35 tests, 35 pass, 0 failed</t>
+          <t>35 node tests pass; plus 15 Playwright checks on the live dashboard DOM</t>
         </is>
       </c>
     </row>
@@ -535,7 +537,19 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Manual cases · Automated Python · Automated Node · Not automatable</t>
+          <t>Coverage · Manual cases · Automated Python · Automated Node · Not automatable</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Coverage</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Python 78% → 99% (2026-09-28, second pass); see Coverage sheet</t>
         </is>
       </c>
     </row>
@@ -545,6 +559,285 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="110" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>File / check</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Before</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>After</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>build_site.py</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>88%</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>99%</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>5 lines: __main__ guard and resolve() guards that cannot raise on Python 3.11</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>validate_site.py</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>85%</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>99%</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>2 lines: unreachable filesystem-root refusal</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>scrape_greenjobs.py</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>18%</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>99%</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>1 line: __main__ guard; crawl replayed from 12 real pages recorded 2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>TOTAL Python</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>78%</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>99%</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>8 of 2,101 statements uncovered</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>lib.js (node)</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>97.7%</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>97.7%</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>two edge branches</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>dashboard.js (node)</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>57.1%</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>57.1% + 15 browser checks</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>DOM half runs in real Chromium (dashboard_dom.test.mjs); node cannot attribute browser-executed lines</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Mutation check: esc() quote=False</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr"/>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>caught</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>7 checks fail in test_gaps, 1 in test_build</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Mutation check: hero budget = 1 byte</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr"/>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>caught</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>8 checks fail</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Mutation check: landing 0-role guard removed</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr"/>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>caught</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>12 checks fail</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Mutation check: snapshot floor 0.5 → 0.1</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr"/>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>caught</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>test_scrape</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Mutation check: € mapped to GBP</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr"/>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>caught</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>test_scrape parse_salary</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Reproduce</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr"/>
+      <c r="C13" s="4" t="inlineStr"/>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>python3 -m coverage run --include="execution/gtm_client_workflows/greenjobs_redesign/*" tests/greenjobs_redesign/test_build.py &amp;&amp; python3 -m coverage report -m</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:D13"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2177,20 +2470,20 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E44"/>
+  <dimension ref="A1:E69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="46" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
     <col width="70" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2201,7 +2494,7 @@
       </c>
       <c r="B1" s="3" t="inlineStr">
         <is>
-          <t>Block</t>
+          <t>File</t>
         </is>
       </c>
       <c r="C1" s="3" t="inlineStr">
@@ -2211,12 +2504,12 @@
       </c>
       <c r="D1" s="3" t="inlineStr">
         <is>
-          <t>Assertions</t>
+          <t>check() calls</t>
         </is>
       </c>
       <c r="E1" s="3" t="inlineStr">
         <is>
-          <t>Line (test_build.py)</t>
+          <t>Line</t>
         </is>
       </c>
     </row>
@@ -2228,15 +2521,15 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>test_build.py</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr"/>
       <c r="D2" s="4" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>44</v>
+        <v>53</v>
       </c>
     </row>
     <row r="3">
@@ -2247,15 +2540,15 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>test_build.py</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr"/>
       <c r="D3" s="4" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>51</v>
+        <v>60</v>
       </c>
     </row>
     <row r="4">
@@ -2266,15 +2559,15 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>test_build.py</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr"/>
       <c r="D4" s="4" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>58</v>
+        <v>67</v>
       </c>
     </row>
     <row r="5">
@@ -2285,15 +2578,15 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>test_build.py</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr"/>
       <c r="D5" s="4" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>68</v>
+        <v>77</v>
       </c>
     </row>
     <row r="6">
@@ -2304,15 +2597,15 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>test_build.py</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr"/>
       <c r="D6" s="4" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>80</v>
+        <v>89</v>
       </c>
     </row>
     <row r="7">
@@ -2323,15 +2616,15 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>test_build.py</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr"/>
       <c r="D7" s="4" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>90</v>
+        <v>99</v>
       </c>
     </row>
     <row r="8">
@@ -2342,15 +2635,15 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>test_build.py</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr"/>
       <c r="D8" s="4" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>96</v>
+        <v>105</v>
       </c>
     </row>
     <row r="9">
@@ -2361,15 +2654,15 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>test_build.py</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr"/>
       <c r="D9" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>109</v>
+        <v>118</v>
       </c>
     </row>
     <row r="10">
@@ -2380,15 +2673,15 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>test_build.py</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr"/>
       <c r="D10" s="4" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>114</v>
+        <v>123</v>
       </c>
     </row>
     <row r="11">
@@ -2399,15 +2692,15 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>test_build.py</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr"/>
       <c r="D11" s="4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>126</v>
+        <v>135</v>
       </c>
     </row>
     <row r="12">
@@ -2418,15 +2711,15 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>test_build.py</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr"/>
       <c r="D12" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>134</v>
+        <v>143</v>
       </c>
     </row>
     <row r="13">
@@ -2437,15 +2730,15 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>test_build.py</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr"/>
       <c r="D13" s="4" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>143</v>
+        <v>152</v>
       </c>
     </row>
     <row r="14">
@@ -2456,15 +2749,15 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>test_build.py</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr"/>
       <c r="D14" s="4" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>150</v>
+        <v>159</v>
       </c>
     </row>
     <row r="15">
@@ -2475,15 +2768,15 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>test_build.py</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr"/>
       <c r="D15" s="4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>160</v>
+        <v>169</v>
       </c>
     </row>
     <row r="16">
@@ -2494,15 +2787,15 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>test_build.py</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr"/>
       <c r="D16" s="4" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>170</v>
+        <v>179</v>
       </c>
     </row>
     <row r="17">
@@ -2513,15 +2806,15 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>test_build.py</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr"/>
       <c r="D17" s="4" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>192</v>
+        <v>201</v>
       </c>
     </row>
     <row r="18">
@@ -2532,15 +2825,15 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>test_build.py</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr"/>
       <c r="D18" s="4" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="E18" s="4" t="n">
-        <v>210</v>
+        <v>219</v>
       </c>
     </row>
     <row r="19">
@@ -2551,15 +2844,15 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>dashboard / Keith round</t>
+          <t>test_build.py</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr"/>
       <c r="D19" s="4" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="E19" s="4" t="n">
-        <v>272</v>
+        <v>281</v>
       </c>
     </row>
     <row r="20">
@@ -2570,15 +2863,15 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>dashboard / Keith round</t>
+          <t>test_build.py</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr"/>
       <c r="D20" s="4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E20" s="4" t="n">
-        <v>308</v>
+        <v>317</v>
       </c>
     </row>
     <row r="21">
@@ -2589,15 +2882,15 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>dashboard / Keith round</t>
+          <t>test_build.py</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr"/>
       <c r="D21" s="4" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="E21" s="4" t="n">
-        <v>323</v>
+        <v>332</v>
       </c>
     </row>
     <row r="22">
@@ -2608,15 +2901,15 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Keith round (B/D/G)</t>
+          <t>test_build.py</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr"/>
       <c r="D22" s="4" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="E22" s="4" t="n">
-        <v>371</v>
+        <v>380</v>
       </c>
     </row>
     <row r="23">
@@ -2627,15 +2920,15 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Keith round (B/D/G)</t>
+          <t>test_build.py</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr"/>
       <c r="D23" s="4" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="E23" s="4" t="n">
-        <v>384</v>
+        <v>393</v>
       </c>
     </row>
     <row r="24">
@@ -2646,15 +2939,15 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Keith round (B/D/G)</t>
+          <t>test_build.py</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr"/>
       <c r="D24" s="4" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="E24" s="4" t="n">
-        <v>399</v>
+        <v>408</v>
       </c>
     </row>
     <row r="25">
@@ -2665,15 +2958,15 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>Keith round (B/D/G)</t>
+          <t>test_build.py</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr"/>
       <c r="D25" s="4" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>416</v>
+        <v>425</v>
       </c>
     </row>
     <row r="26">
@@ -2684,15 +2977,15 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>Keith round (B/D/G)</t>
+          <t>test_build.py</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr"/>
       <c r="D26" s="4" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="E26" s="4" t="n">
-        <v>432</v>
+        <v>441</v>
       </c>
     </row>
     <row r="27">
@@ -2703,15 +2996,15 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>Keith round (B/D/G)</t>
+          <t>test_build.py</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr"/>
       <c r="D27" s="4" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="E27" s="4" t="n">
-        <v>458</v>
+        <v>467</v>
       </c>
     </row>
     <row r="28">
@@ -2722,15 +3015,15 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>Keith round (B/D/G)</t>
+          <t>test_build.py</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr"/>
       <c r="D28" s="4" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="E28" s="4" t="n">
-        <v>480</v>
+        <v>489</v>
       </c>
     </row>
     <row r="29">
@@ -2741,15 +3034,15 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>panel fixes A</t>
+          <t>test_build.py</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr"/>
       <c r="D29" s="4" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E29" s="4" t="n">
-        <v>513</v>
+        <v>522</v>
       </c>
     </row>
     <row r="30">
@@ -2760,15 +3053,15 @@
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>panel fixes A</t>
+          <t>test_build.py</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr"/>
       <c r="D30" s="4" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="E30" s="4" t="n">
-        <v>522</v>
+        <v>531</v>
       </c>
     </row>
     <row r="31">
@@ -2779,15 +3072,15 @@
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>panel fixes A</t>
+          <t>test_build.py</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr"/>
       <c r="D31" s="4" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="E31" s="4" t="n">
-        <v>547</v>
+        <v>556</v>
       </c>
     </row>
     <row r="32">
@@ -2798,15 +3091,15 @@
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>panel fixes A</t>
+          <t>test_build.py</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr"/>
       <c r="D32" s="4" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E32" s="4" t="n">
-        <v>562</v>
+        <v>571</v>
       </c>
     </row>
     <row r="33">
@@ -2817,15 +3110,15 @@
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>panel fixes A</t>
+          <t>test_build.py</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr"/>
       <c r="D33" s="4" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="E33" s="4" t="n">
-        <v>595</v>
+        <v>604</v>
       </c>
     </row>
     <row r="34">
@@ -2836,15 +3129,15 @@
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>panel fixes A</t>
+          <t>test_build.py</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr"/>
       <c r="D34" s="4" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="E34" s="4" t="n">
-        <v>622</v>
+        <v>631</v>
       </c>
     </row>
     <row r="35">
@@ -2855,15 +3148,15 @@
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>panel fixes A</t>
+          <t>test_build.py</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr"/>
       <c r="D35" s="4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E35" s="4" t="n">
-        <v>633</v>
+        <v>642</v>
       </c>
     </row>
     <row r="36">
@@ -2874,15 +3167,15 @@
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>panel fixes A</t>
+          <t>test_build.py</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr"/>
       <c r="D36" s="4" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E36" s="4" t="n">
-        <v>644</v>
+        <v>653</v>
       </c>
     </row>
     <row r="37">
@@ -2893,15 +3186,15 @@
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>panel fixes A</t>
+          <t>test_build.py</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr"/>
       <c r="D37" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E37" s="4" t="n">
-        <v>671</v>
+        <v>680</v>
       </c>
     </row>
     <row r="38">
@@ -2912,15 +3205,15 @@
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>panel fixes A</t>
+          <t>test_build.py</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr"/>
       <c r="D38" s="4" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="E38" s="4" t="n">
-        <v>684</v>
+        <v>693</v>
       </c>
     </row>
     <row r="39">
@@ -2931,15 +3224,15 @@
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>panel fixes A</t>
+          <t>test_build.py</t>
         </is>
       </c>
       <c r="C39" s="4" t="inlineStr"/>
       <c r="D39" s="4" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E39" s="4" t="n">
-        <v>705</v>
+        <v>714</v>
       </c>
     </row>
     <row r="40">
@@ -2950,15 +3243,15 @@
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>panel fixes A</t>
+          <t>test_build.py</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr"/>
       <c r="D40" s="4" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="E40" s="4" t="n">
-        <v>720</v>
+        <v>729</v>
       </c>
     </row>
     <row r="41">
@@ -2969,15 +3262,15 @@
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>panel fixes A</t>
+          <t>test_build.py</t>
         </is>
       </c>
       <c r="C41" s="4" t="inlineStr"/>
       <c r="D41" s="4" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E41" s="4" t="n">
-        <v>760</v>
+        <v>769</v>
       </c>
     </row>
     <row r="42">
@@ -2988,15 +3281,15 @@
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>panel fixes A</t>
+          <t>test_build.py</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr"/>
       <c r="D42" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E42" s="4" t="n">
-        <v>771</v>
+        <v>780</v>
       </c>
     </row>
     <row r="43">
@@ -3007,15 +3300,15 @@
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>panel fixes B</t>
+          <t>test_build.py</t>
         </is>
       </c>
       <c r="C43" s="4" t="inlineStr"/>
       <c r="D43" s="4" t="n">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="E43" s="4" t="n">
-        <v>845</v>
+        <v>862</v>
       </c>
     </row>
     <row r="44">
@@ -3026,7 +3319,7 @@
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>panel fixes B</t>
+          <t>test_build.py</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
@@ -3035,19 +3328,498 @@
         </is>
       </c>
       <c r="D44" s="4" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E44" s="4" t="n">
-        <v>936</v>
+        <v>953</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>test_parse_salary</t>
+        </is>
+      </c>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>test_scrape.py (recorded corpus)</t>
+        </is>
+      </c>
+      <c r="C45" s="4" t="inlineStr"/>
+      <c r="D45" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="E45" s="4" t="n">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>test_text_helpers</t>
+        </is>
+      </c>
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>test_scrape.py (recorded corpus)</t>
+        </is>
+      </c>
+      <c r="C46" s="4" t="inlineStr"/>
+      <c r="D46" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="E46" s="4" t="n">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>test_parse_results_and_facets</t>
+        </is>
+      </c>
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>test_scrape.py (recorded corpus)</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="inlineStr"/>
+      <c r="D47" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="E47" s="4" t="n">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>test_parse_job_fields</t>
+        </is>
+      </c>
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>test_scrape.py (recorded corpus)</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="inlineStr"/>
+      <c r="D48" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="E48" s="4" t="n">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>test_measure_page</t>
+        </is>
+      </c>
+      <c r="B49" s="4" t="inlineStr">
+        <is>
+          <t>test_scrape.py (recorded corpus)</t>
+        </is>
+      </c>
+      <c r="C49" s="4" t="inlineStr"/>
+      <c r="D49" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E49" s="4" t="n">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>test_fetch_error_branches</t>
+        </is>
+      </c>
+      <c r="B50" s="4" t="inlineStr">
+        <is>
+          <t>test_scrape.py (recorded corpus)</t>
+        </is>
+      </c>
+      <c r="C50" s="4" t="inlineStr"/>
+      <c r="D50" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="E50" s="4" t="n">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>test_snapshot_floor_and_atomic_write</t>
+        </is>
+      </c>
+      <c r="B51" s="4" t="inlineStr">
+        <is>
+          <t>test_scrape.py (recorded corpus)</t>
+        </is>
+      </c>
+      <c r="C51" s="4" t="inlineStr"/>
+      <c r="D51" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="E51" s="4" t="n">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>test_crawl_ie</t>
+        </is>
+      </c>
+      <c r="B52" s="4" t="inlineStr">
+        <is>
+          <t>test_scrape.py (recorded corpus)</t>
+        </is>
+      </c>
+      <c r="C52" s="4" t="inlineStr"/>
+      <c r="D52" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="E52" s="4" t="n">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>test_crawl_uk_with_logos_and_paging</t>
+        </is>
+      </c>
+      <c r="B53" s="4" t="inlineStr">
+        <is>
+          <t>test_scrape.py (recorded corpus)</t>
+        </is>
+      </c>
+      <c r="C53" s="4" t="inlineStr"/>
+      <c r="D53" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="E53" s="4" t="n">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>test_crawl_paging_and_missing_page</t>
+        </is>
+      </c>
+      <c r="B54" s="4" t="inlineStr">
+        <is>
+          <t>test_scrape.py (recorded corpus)</t>
+        </is>
+      </c>
+      <c r="C54" s="4" t="inlineStr"/>
+      <c r="D54" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E54" s="4" t="n">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>test_snapshot_floor_rejects_and_main_exit_code</t>
+        </is>
+      </c>
+      <c r="B55" s="4" t="inlineStr">
+        <is>
+          <t>test_scrape.py (recorded corpus)</t>
+        </is>
+      </c>
+      <c r="C55" s="4" t="inlineStr"/>
+      <c r="D55" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E55" s="4" t="n">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>test_homepage_snapshot_fallback</t>
+        </is>
+      </c>
+      <c r="B56" s="4" t="inlineStr">
+        <is>
+          <t>test_scrape.py (recorded corpus)</t>
+        </is>
+      </c>
+      <c r="C56" s="4" t="inlineStr"/>
+      <c r="D56" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="E56" s="4" t="n">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>test_fixture_provenance</t>
+        </is>
+      </c>
+      <c r="B57" s="4" t="inlineStr">
+        <is>
+          <t>test_scrape.py (recorded corpus)</t>
+        </is>
+      </c>
+      <c r="C57" s="4" t="inlineStr"/>
+      <c r="D57" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E57" s="4" t="n">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>test_helper_edges</t>
+        </is>
+      </c>
+      <c r="B58" s="4" t="inlineStr">
+        <is>
+          <t>test_gaps.py (branch tests)</t>
+        </is>
+      </c>
+      <c r="C58" s="4" t="inlineStr"/>
+      <c r="D58" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="E58" s="4" t="n">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="4" t="inlineStr">
+        <is>
+          <t>test_dataset_and_brief</t>
+        </is>
+      </c>
+      <c r="B59" s="4" t="inlineStr">
+        <is>
+          <t>test_gaps.py (branch tests)</t>
+        </is>
+      </c>
+      <c r="C59" s="4" t="inlineStr"/>
+      <c r="D59" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="E59" s="4" t="n">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="4" t="inlineStr">
+        <is>
+          <t>test_hero_footage_variants</t>
+        </is>
+      </c>
+      <c r="B60" s="4" t="inlineStr">
+        <is>
+          <t>test_gaps.py (branch tests)</t>
+        </is>
+      </c>
+      <c r="C60" s="4" t="inlineStr"/>
+      <c r="D60" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="E60" s="4" t="n">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="4" t="inlineStr">
+        <is>
+          <t>test_geometry_helpers</t>
+        </is>
+      </c>
+      <c r="B61" s="4" t="inlineStr">
+        <is>
+          <t>test_gaps.py (branch tests)</t>
+        </is>
+      </c>
+      <c r="C61" s="4" t="inlineStr">
+        <is>
+          <t>svg_polygons / ring_area / point_in_rings / sample_map_points / film_payload</t>
+        </is>
+      </c>
+      <c r="D61" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="E61" s="4" t="n">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="4" t="inlineStr">
+        <is>
+          <t>test_escaping_in_rendered_html</t>
+        </is>
+      </c>
+      <c r="B62" s="4" t="inlineStr">
+        <is>
+          <t>test_gaps.py (branch tests)</t>
+        </is>
+      </c>
+      <c r="C62" s="4" t="inlineStr"/>
+      <c r="D62" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="E62" s="4" t="n">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="4" t="inlineStr">
+        <is>
+          <t>test_landing_zero_role_guard</t>
+        </is>
+      </c>
+      <c r="B63" s="4" t="inlineStr">
+        <is>
+          <t>test_gaps.py (branch tests)</t>
+        </is>
+      </c>
+      <c r="C63" s="4" t="inlineStr"/>
+      <c r="D63" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="E63" s="4" t="n">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="4" t="inlineStr">
+        <is>
+          <t>test_node_and_js_checks</t>
+        </is>
+      </c>
+      <c r="B64" s="4" t="inlineStr">
+        <is>
+          <t>test_gaps.py (branch tests)</t>
+        </is>
+      </c>
+      <c r="C64" s="4" t="inlineStr"/>
+      <c r="D64" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="E64" s="4" t="n">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="4" t="inlineStr">
+        <is>
+          <t>test_guard_output_edges</t>
+        </is>
+      </c>
+      <c r="B65" s="4" t="inlineStr">
+        <is>
+          <t>test_gaps.py (branch tests)</t>
+        </is>
+      </c>
+      <c r="C65" s="4" t="inlineStr"/>
+      <c r="D65" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E65" s="4" t="n">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="4" t="inlineStr">
+        <is>
+          <t>test_build_failure_exits</t>
+        </is>
+      </c>
+      <c r="B66" s="4" t="inlineStr">
+        <is>
+          <t>test_gaps.py (branch tests)</t>
+        </is>
+      </c>
+      <c r="C66" s="4" t="inlineStr"/>
+      <c r="D66" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="E66" s="4" t="n">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="4" t="inlineStr">
+        <is>
+          <t>test_rebuild_and_no_site_base</t>
+        </is>
+      </c>
+      <c r="B67" s="4" t="inlineStr">
+        <is>
+          <t>test_gaps.py (branch tests)</t>
+        </is>
+      </c>
+      <c r="C67" s="4" t="inlineStr"/>
+      <c r="D67" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="E67" s="4" t="n">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="4" t="inlineStr">
+        <is>
+          <t>test_cli_main_with_today</t>
+        </is>
+      </c>
+      <c r="B68" s="4" t="inlineStr">
+        <is>
+          <t>test_gaps.py (branch tests)</t>
+        </is>
+      </c>
+      <c r="C68" s="4" t="inlineStr"/>
+      <c r="D68" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E68" s="4" t="n">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="4" t="inlineStr">
+        <is>
+          <t>test_validator_every_message</t>
+        </is>
+      </c>
+      <c r="B69" s="4" t="inlineStr">
+        <is>
+          <t>test_gaps.py (branch tests)</t>
+        </is>
+      </c>
+      <c r="C69" s="4" t="inlineStr"/>
+      <c r="D69" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="E69" s="4" t="n">
+        <v>383</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E44"/>
+  <autoFilter ref="A1:E69"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3498,7 +4270,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
[greenjobs] Round-3 fixes (package table height, IE employer count wording, long dates, filter rail, map zero regions, NI at 390, agency casing, secondary tags, unverified salary source, hero CTA, marquee logos, monogram tiles); re-verified requirements matrix v2 + visual sweep v2; spreadsheet gains Keith requirements sheet
Co-Authored-By: Claude <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XyZXNeMjVmnqRyKctLtDmB
</commit_message>
<xml_diff>
--- a/deliverables/greenjobs_redesign_2026-09-22/tests_register_2026-09-28.xlsx
+++ b/deliverables/greenjobs_redesign_2026-09-22/tests_register_2026-09-28.xlsx
@@ -8,18 +8,20 @@
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Coverage" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Manual cases" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Automated Python" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Automated Node" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Not automatable" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Keith requirements" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Coverage" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Manual cases" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Automated Python" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Automated Node" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Not automatable" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Coverage'!$A$1:$D$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Manual cases'!$A$1:$G$46</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Automated Python'!$A$1:$E$69</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Automated Node'!$A$1:$B$36</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Not automatable'!$A$1:$C$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Keith requirements'!$A$1:$H$115</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Coverage'!$A$1:$D$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Manual cases'!$A$1:$G$46</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Automated Python'!$A$1:$E$69</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Automated Node'!$A$1:$B$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Not automatable'!$A$1:$C$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -48,7 +50,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -58,6 +60,31 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="002F5D3A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E3F1E3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FDE9D9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF3CD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2E3F5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8D7DA"/>
       </patternFill>
     </fill>
   </fills>
@@ -73,7 +100,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -81,6 +108,21 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -448,7 +490,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -553,12 +595,4135 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Keith's document, sentence by sentence (114 rows, re-verified on the final build)</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>DONE: 96, INTERPRETED DIFFERENTLY: 3, PARTIAL: 7, NEEDS CLIENT INPUT: 7, NOT DONE: 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Visual sweep (32 issues found by a picky pass + 6 found on re-check)</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>All fixable ones fixed and re-screenshotted; see research/qa_2026-09-28/visual_issues_v2.md</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H115"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="70" customWidth="1" min="6" max="6"/>
+    <col width="60" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>requirement_verbatim</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>edition</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>evidence</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>delta</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>changed_since_v1</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>R001</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>Proposition</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>“Work that puts the planet on the payroll” is memorable, but slightly abstract. I prefer: Work that works for the planet or Build your career. Protect our future.</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>IE+UK</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>/ie/ and /uk/ hero h1 text = "Work that works for the planet." (grep ie/index.html, uk/index.html; shots ie_home_1440_light, uk_home_1440_dark)</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr"/>
+      <c r="H2" s="5" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>R002</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Proposition</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>Find environmental, sustainability, renewable-energy and nature careers across Ireland.</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>IE</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>/ie/ hero subheading is the exact sentence (ie/index.html text dump)</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr"/>
+      <c r="H3" s="5" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>R003</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Remove “3 employers”</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Remove “3 employers” from the hero</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>IE</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>/ie/ hero strip = "88 live roles · Specialist green job network since 2008 · 10 specialist job sites · Roles across 14 sectors · Snapshot of 22 September 2026"; no employer count in the strip</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>Count still appears lower on /ie/ and /ie/employers/: "3 of them have live roles on greenjobs.ie this week" (grep "3 of them")</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>R004</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Remove “3 employers”</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Specialist green job network since 2008</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>IE+UK</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>Both hero strips contain "Specialist green job network since 2008"</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr"/>
+      <c r="H5" s="5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>R005</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Remove “3 employers”</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>10 specialist job sites</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>IE+UK</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>Both hero strips contain "10 specialist job sites"</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr"/>
+      <c r="H6" s="5" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>R006</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>Remove “3 employers”</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>Roles across 10 sectors</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>IE+UK</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>INTERPRETED DIFFERENTLY</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>Hero strip now reads "Roles across 14 sectors" on both editions (was 15/14); computed from sectors with &gt;=1 live role</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>Client wrote 10; site shows the live count 14. Still needs the client to confirm which number</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>R007</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Remove “3 employers”</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Certified B Corporation</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>IE+UK</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>Header badge now has a text label "Certified B Corp" (span.hdr__bcorp) + hero pill "Certified B Corporation. Independently verified for…" on both editions (crop ie_home_hero)</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>Label added since v1</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>R008</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Classification</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Road engineering and infrastructure roles appear under “Sustainability &amp; net zero.”</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>IE+UK</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>"Sustainability &amp; net zero" appears in no page except the for-keith evidence quote; Assistant Road Engineer / Highways Civil Engineer tagged "Sustainable infrastructure &amp; transport" only (jobs.json)</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr"/>
+      <c r="H9" s="5" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>R009</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>Classification</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>UK-only roles also appear prominently on the Irish board with salaries converted into euros.</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>IE</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>INTERPRETED DIFFERENTLY</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>Per Keith's 28-Sept rule (KEITH_CHANGES_CHECKLIST B5) the IE board keeps UK-only roles, labelled "UK", with the toggle doing the excluding. jobs.json IE: 62 ie / 23 uk / 3 cross; 21 of the 23 UK roles now show advertised sterling "£62k–67k (paid in sterling, about €72.5k–78.4k)" (/ie/ first card, /ie/jobs/11501460/)</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>Was NOT DONE. Prominence is now a client decision; 2 UK-only roles (11497629 Associate Civil Engineer London €70–75k, 11496364 Planner Scotland €30–40k) still carry euro figures with no "Salary source" row</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="inlineStr">
+        <is>
+          <t>NOT DONE → INTERPRETED DIFFERENTLY</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>R010</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Classification</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>Improve sector mapping.</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>IE+UK</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>14-sector taxonomy; Highways Civil Engineer (uk 11501402) and Assistant Road Engineer now single-tagged infrastructure; Design Coordinator – Rail, Principal Engineer – Transportation, Civil Engineering Technician all "Sustainable infrastructure &amp; transport"</t>
+        </is>
+      </c>
+      <c r="G11" s="7" t="inlineStr">
+        <is>
+          <t>Associate Civil Engineer (ie 11497629) still also tagged "Built environment &amp; energy efficiency"; Principal Project Manager – Civil &amp; Environmental sits under Environmental engineering + Waste</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>R011</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Classification</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>Retain salaries in their original advertised currency.</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>IE+UK</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>UK: /uk/jobs/11501639/ "€5.1k–6k/mo (paid in euros, about £4.4k–5.1k/mo)". IE: /ie/jobs/11500760/ Salary "£45,000 to £55,000 per annum (paid in sterling, about €52.7k–64.3k)" + "Salary source: Advertised in sterling on the greenjobs.co.uk listing"; IE jobs.json cur: 21 GBP, 8 EUR, 59 none</t>
+        </is>
+      </c>
+      <c r="G12" s="7" t="inlineStr">
+        <is>
+          <t>Improved: 21/23 IE sterling roles restored. 2 UK-located roles (11497629, 11496364) still show € figures; scraped from greenjobs.ie with no UK twin, so the original currency is unverified</t>
+        </is>
+      </c>
+      <c r="H12" s="7" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>R012</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Classification</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Clearly label UK, Ireland, remote and cross-border positions.</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>IE+UK</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>Chips "UK", "Ireland", "Ireland &amp; UK", "Remote"; Commonland roles now "Dublin · Ireland &amp; UK" on /ie/ and /ie/jobs/ (was "Dublin · Ireland"); /ie/jobs/11500760/ facts panel "Where: UK"</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>Cross-border labelling fixed since v1</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>PARTIAL → DONE</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>R013</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Classification</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Allow users to exclude UK opportunities.</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>IE</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>/ie/jobs/ checkbox "Hide UK/abroad-only roles — Keeps Ireland, Northern Ireland, remote and Ireland-and-UK roles; hides roles advertised only in the UK or abroad."</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr"/>
+      <c r="H14" s="5" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>R014</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Classification</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Explain when one job appears in multiple counties or sectors, as totals otherwise look inconsistent.</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>IE+UK</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>/ie/ "A role listed in more than one county or sector counts in each; salary figures use the midpoint…"; /ie/jobs/, /ie/sectors/, salary guide carry the same note</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr"/>
+      <c r="H15" s="5" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>R015</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Shorten the homepage</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>County information appears twice.</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>IE</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>/ie/ has one county mention: stat tile "14 counties with live roles"; no county map on home</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr"/>
+      <c r="H16" s="5" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>R016</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Shorten the homepage</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Sector information appears twice.</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>IE+UK</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>One "Browse by sector" section per home page (9 cards + "All sectors")</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="inlineStr"/>
+      <c r="H17" s="5" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>R017</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Shorten the homepage</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Salary transparency appears in several places.</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>IE+UK</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>One "Salary insight" section per home; sector cards carry only a median/disclosure line</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr"/>
+      <c r="H18" s="5" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>R018</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Shorten the homepage</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>The CV-matching tool is repeated on the jobs page.</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>IE+UK</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>"Quick job match" only on /ie/jobs/ and /uk/jobs/ (grep home pages: 0)</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="inlineStr"/>
+      <c r="H19" s="5" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>R019</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Shorten the homepage</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>A simpler sequence would be: Hero and search</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>IE</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>/ie/ order: hero+search → Latest roles → Browse by sector → Salary insight → Why GreenJobs → Employer proposition → Email alerts (text dump)</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="inlineStr"/>
+      <c r="H20" s="5" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>R020</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Shorten the homepage</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>Featured/latest roles</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>IE</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>/ie/ "Latest roles" (8 cards) second</t>
+        </is>
+      </c>
+      <c r="G21" s="5" t="inlineStr"/>
+      <c r="H21" s="5" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>R021</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Shorten the homepage</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>Browse by sector</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>IE</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>/ie/ "Browse by sector" third</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="inlineStr"/>
+      <c r="H22" s="5" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>R022</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>Shorten the homepage</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>Salary insight</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>IE</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>/ie/ "Salary insight" fourth</t>
+        </is>
+      </c>
+      <c r="G23" s="5" t="inlineStr"/>
+      <c r="H23" s="5" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>R023</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>Shorten the homepage</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>Why GreenJobs</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>IE</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="inlineStr">
+        <is>
+          <t>/ie/ "Why GreenJobs" fifth</t>
+        </is>
+      </c>
+      <c r="G24" s="5" t="inlineStr"/>
+      <c r="H24" s="5" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>R024</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>Shorten the homepage</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>Employer proposition</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>IE</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>/ie/ "Employer proposition" sixth</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="inlineStr"/>
+      <c r="H25" s="5" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>R025</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Shorten the homepage</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>Email alerts</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>IE</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>/ie/ "Email alerts: the week's green roles, in your inbox" last</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="inlineStr"/>
+      <c r="H26" s="5" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>R026</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>Shorten the homepage</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>The interactive data elements are good, but there are currently too many competing for attention.</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>IE+UK</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F27" s="5" t="inlineStr">
+        <is>
+          <t>IE home: sector sparklines + 3 stat tiles; UK home: one region map + 3 stat tiles (shots ie_home_1440_light, uk_home_1440_dark)</t>
+        </is>
+      </c>
+      <c r="G27" s="5" t="inlineStr"/>
+      <c r="H27" s="5" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>R027</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Candidate experience</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>Workplace type: office, hybrid, remote or site-based</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>IE+UK</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F28" s="5" t="inlineStr">
+        <is>
+          <t>/uk/jobs/ Workplace: Office-based, Hybrid, Remote, Site-based, Not stated; /ie/jobs/ omits Office-based (jobs.json IE has 0 office roles)</t>
+        </is>
+      </c>
+      <c r="G28" s="5" t="inlineStr"/>
+      <c r="H28" s="5" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>R028</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>Candidate experience</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>Career level</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t>IE+UK</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>Career level select: Graduate/Early career, Mid-level, Senior/Principal, Director/Associate (both editions)</t>
+        </is>
+      </c>
+      <c r="G29" s="5" t="inlineStr"/>
+      <c r="H29" s="5" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>R029</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>Candidate experience</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>Salary range</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>IE+UK</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F30" s="5" t="inlineStr">
+        <is>
+          <t>"Salary, EUR/GBP a year" Minimum/Maximum + "Salary disclosed only" + note "Ranges are compared per year in EUR; every role still shows the salary in the currency it was advertised in."</t>
+        </is>
+      </c>
+      <c r="G30" s="5" t="inlineStr"/>
+      <c r="H30" s="5" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>R030</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>Candidate experience</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>Permanent, contract, fixed-term, full-time and part-time</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>IE+UK</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F31" s="5" t="inlineStr">
+        <is>
+          <t>Single "Contract" select: Permanent, Contract, Fixed-term, Full-time (+Part-time, Volunteer on UK). The overlapping "Job type" select is gone (grep "Job type": 0)</t>
+        </is>
+      </c>
+      <c r="G31" s="5" t="inlineStr">
+        <is>
+          <t>Duplicate select removed since v1</t>
+        </is>
+      </c>
+      <c r="H31" s="5" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>R031</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>Candidate experience</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>Ireland-only toggle</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>IE</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F32" s="5" t="inlineStr">
+        <is>
+          <t>/ie/jobs/ "Hide UK/abroad-only roles" checkbox</t>
+        </is>
+      </c>
+      <c r="G32" s="5" t="inlineStr"/>
+      <c r="H32" s="5" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>R032</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>Candidate experience</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>Closing date</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>IE+UK</t>
+        </is>
+      </c>
+      <c r="E33" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F33" s="5" t="inlineStr">
+        <is>
+          <t>Closing date select: Any / within 7 / 14 / 30 days + "Hide closed roles"</t>
+        </is>
+      </c>
+      <c r="G33" s="5" t="inlineStr"/>
+      <c r="H33" s="5" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>R033</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>Candidate experience</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>Direct employer versus recruitment agency</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>IE+UK</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F34" s="5" t="inlineStr">
+        <is>
+          <t>"Advertised by": Employers and agencies / Direct employer / Recruitment agency; job pages show "Advertised by: Recruitment agency"</t>
+        </is>
+      </c>
+      <c r="G34" s="5" t="inlineStr"/>
+      <c r="H34" s="5" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>R034</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>Candidate experience</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>“Similar jobs” on individual vacancy pages</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="inlineStr">
+        <is>
+          <t>IE+UK</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F35" s="5" t="inlineStr">
+        <is>
+          <t>/ie/jobs/11500760/, /ie/jobs/11501460/, /uk/jobs/11501639/, /uk/jobs/11501402/ each have "Similar roles — Same sector first, then the same area, then similar pay" with 4 cards</t>
+        </is>
+      </c>
+      <c r="G35" s="5" t="inlineStr"/>
+      <c r="H35" s="5" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>R035</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>Candidate experience</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>Rename “Your fit in ten seconds” to something more credible, such as Quick job match.</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>IE+UK</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F36" s="5" t="inlineStr">
+        <is>
+          <t>h2 "Quick job match" on both jobs pages; "Your fit in ten seconds" only in the for-keith quote</t>
+        </is>
+      </c>
+      <c r="G36" s="5" t="inlineStr"/>
+      <c r="H36" s="5" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>R036</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>Candidate experience</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>Put this directly beside the input: Your information is processed on your device and is not uploaded or stored.</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>IE+UK</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F37" s="5" t="inlineStr">
+        <is>
+          <t>Both jobs pages: "Your information is processed on your device and is not uploaded or stored." rendered in bold beside (right of) the textarea at 1440 (crop ie_jobsmap_top)</t>
+        </is>
+      </c>
+      <c r="G37" s="5" t="inlineStr">
+        <is>
+          <t>Exact sentence and placement fixed since v1</t>
+        </is>
+      </c>
+      <c r="H37" s="5" t="inlineStr">
+        <is>
+          <t>PARTIAL → DONE</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>R037</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>Candidate experience</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>Also make clear that it is keyword matching, not a formal assessment of someone’s suitability.</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>IE+UK</t>
+        </is>
+      </c>
+      <c r="E38" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F38" s="5" t="inlineStr">
+        <is>
+          <t>Directly under it: "Keyword matching, not an assessment of your suitability."</t>
+        </is>
+      </c>
+      <c r="G38" s="5" t="inlineStr"/>
+      <c r="H38" s="5" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>R038</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>Employer conversion</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>Actual prices or a clear “Request advertising rates” CTA</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="inlineStr">
+        <is>
+          <t>IE+UK</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F39" s="5" t="inlineStr">
+        <is>
+          <t>/ie/employers/ and /uk/employers/: "Request advertising rates →" in hero, above the table and in the form; "Prices are not published. Rates are supplied by the team…"</t>
+        </is>
+      </c>
+      <c r="G39" s="5" t="inlineStr"/>
+      <c r="H39" s="5" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="8" t="inlineStr">
+        <is>
+          <t>R039</t>
+        </is>
+      </c>
+      <c r="B40" s="8" t="inlineStr">
+        <is>
+          <t>Employer conversion</t>
+        </is>
+      </c>
+      <c r="C40" s="8" t="inlineStr">
+        <is>
+          <t>Candidate audience and newsletter reach</t>
+        </is>
+      </c>
+      <c r="D40" s="8" t="inlineStr">
+        <is>
+          <t>IE+UK</t>
+        </is>
+      </c>
+      <c r="E40" s="8" t="inlineStr">
+        <is>
+          <t>NEEDS CLIENT INPUT</t>
+        </is>
+      </c>
+      <c r="F40" s="8" t="inlineStr">
+        <is>
+          <t>"Audience and reach" block reads "Thousands of visitors every month…" then "Monthly visitor figures are published at launch." / "Subscriber numbers are published at launch."</t>
+        </is>
+      </c>
+      <c r="G40" s="8" t="inlineStr">
+        <is>
+          <t>Placeholder wording softened but figures still missing; client must supply</t>
+        </is>
+      </c>
+      <c r="H40" s="8" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="8" t="inlineStr">
+        <is>
+          <t>R040</t>
+        </is>
+      </c>
+      <c r="B41" s="8" t="inlineStr">
+        <is>
+          <t>Employer conversion</t>
+        </is>
+      </c>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>LinkedIn and network distribution figures</t>
+        </is>
+      </c>
+      <c r="D41" s="8" t="inlineStr">
+        <is>
+          <t>IE+UK</t>
+        </is>
+      </c>
+      <c r="E41" s="8" t="inlineStr">
+        <is>
+          <t>NEEDS CLIENT INPUT</t>
+        </is>
+      </c>
+      <c r="F41" s="8" t="inlineStr">
+        <is>
+          <t>"Network and LinkedIn distribution" ends "Network and follower numbers are published at launch."</t>
+        </is>
+      </c>
+      <c r="G41" s="8" t="inlineStr">
+        <is>
+          <t>Client must supply</t>
+        </is>
+      </c>
+      <c r="H41" s="8" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="7" t="inlineStr">
+        <is>
+          <t>R041</t>
+        </is>
+      </c>
+      <c r="B42" s="7" t="inlineStr">
+        <is>
+          <t>Employer conversion</t>
+        </is>
+      </c>
+      <c r="C42" s="7" t="inlineStr">
+        <is>
+          <t>Examples of organisations that have recruited through GreenJobs</t>
+        </is>
+      </c>
+      <c r="D42" s="7" t="inlineStr">
+        <is>
+          <t>IE+UK</t>
+        </is>
+      </c>
+      <c r="E42" s="7" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="F42" s="7" t="inlineStr">
+        <is>
+          <t>UK: 12 logo tiles in the marquee (Arup, Commonland, Dacorum, ESS, Gaia, Grundon, Haskoning, Jacobs…). IE: Mattinson logo + text-only tiles "Commonland", "Gaia Talent" (crop ie_home_employers); EirGrid/Power NI/Veolia dropped</t>
+        </is>
+      </c>
+      <c r="G42" s="7" t="inlineStr">
+        <is>
+          <t>IE tiles still text-only; only organisations with live roles are shown now</t>
+        </is>
+      </c>
+      <c r="H42" s="7" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>R042</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>Employer conversion</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>A comparison table for Standard, Premium and Membership packages</t>
+        </is>
+      </c>
+      <c r="D43" s="5" t="inlineStr">
+        <is>
+          <t>IE+UK</t>
+        </is>
+      </c>
+      <c r="E43" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F43" s="5" t="inlineStr">
+        <is>
+          <t>"Compare the options" table renders as a proper 4-column grid with green "Included" ticks and muted "Ask us" (crop ie_emp_table); at 390 it collapses to one card per row (crop ie_emp390_table)</t>
+        </is>
+      </c>
+      <c r="G43" s="5" t="inlineStr">
+        <is>
+          <t>Rendering fixed since v1. New defect: .cmpwrap max-height 648px hides the last two rows (the Membership "Included" rows) at 1440×900 with no scroll cue — see visual_issues_v2 N1</t>
+        </is>
+      </c>
+      <c r="H43" s="5" t="inlineStr">
+        <is>
+          <t>PARTIAL → DONE</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="7" t="inlineStr">
+        <is>
+          <t>R043</t>
+        </is>
+      </c>
+      <c r="B44" s="7" t="inlineStr">
+        <is>
+          <t>Employer conversion</t>
+        </is>
+      </c>
+      <c r="C44" s="7" t="inlineStr">
+        <is>
+          <t>“Employer branding” and “Packages and memberships” currently feel like headings rather than fully developed products.</t>
+        </is>
+      </c>
+      <c r="D44" s="7" t="inlineStr">
+        <is>
+          <t>IE+UK</t>
+        </is>
+      </c>
+      <c r="E44" s="7" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="F44" s="7" t="inlineStr">
+        <is>
+          <t>Headings replaced by "Audience and reach", "Compare the options", "Post a job"; Membership column is 11×"Ask us" + 2 Included</t>
+        </is>
+      </c>
+      <c r="G44" s="7" t="inlineStr">
+        <is>
+          <t>Products remain thin; needs client content</t>
+        </is>
+      </c>
+      <c r="H44" s="7" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>R044</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t>Employer conversion</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>The live site should concentrate on the outcome: Preview exactly how your vacancy will appear to candidates.</t>
+        </is>
+      </c>
+      <c r="D45" s="5" t="inlineStr">
+        <is>
+          <t>IE+UK</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F45" s="5" t="inlineStr">
+        <is>
+          <t>Lede "Preview exactly how your vacancy will appear to candidates."; remaining form note is "Preview only. Rates and posting are handled by the GreenJobs team." (no "Posting opens at launch", grep 0)</t>
+        </is>
+      </c>
+      <c r="G45" s="5" t="inlineStr">
+        <is>
+          <t>Launch disclaimer removed since v1</t>
+        </is>
+      </c>
+      <c r="H45" s="5" t="inlineStr">
+        <is>
+          <t>PARTIAL → DONE</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>R045</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="inlineStr">
+        <is>
+          <t>Copy and credibility</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>“Career level read from title”</t>
+        </is>
+      </c>
+      <c r="D46" s="5" t="inlineStr">
+        <is>
+          <t>IE+UK</t>
+        </is>
+      </c>
+      <c r="E46" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F46" s="5" t="inlineStr">
+        <is>
+          <t>grep across site HTML: only in for-keith evidence quote (noindex)</t>
+        </is>
+      </c>
+      <c r="G46" s="5" t="inlineStr"/>
+      <c r="H46" s="5" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>R046</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>Copy and credibility</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>“Tagged by what its description actually says”</t>
+        </is>
+      </c>
+      <c r="D47" s="5" t="inlineStr">
+        <is>
+          <t>IE+UK</t>
+        </is>
+      </c>
+      <c r="E47" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F47" s="5" t="inlineStr">
+        <is>
+          <t>grep: only in for-keith quote; dashboard says "each role is tagged to the sectors its description talks about"</t>
+        </is>
+      </c>
+      <c r="G47" s="5" t="inlineStr"/>
+      <c r="H47" s="5" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>R047</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t>Copy and credibility</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>“The send button is honest”</t>
+        </is>
+      </c>
+      <c r="D48" s="5" t="inlineStr">
+        <is>
+          <t>IE+UK</t>
+        </is>
+      </c>
+      <c r="E48" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F48" s="5" t="inlineStr">
+        <is>
+          <t>grep: only in for-keith quote</t>
+        </is>
+      </c>
+      <c r="G48" s="5" t="inlineStr"/>
+      <c r="H48" s="5" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>R048</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="inlineStr">
+        <is>
+          <t>Copy and credibility</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>Replace this with benefit-led language: Every vacancy is classified consistently, making it easier to compare roles, sectors and salaries.</t>
+        </is>
+      </c>
+      <c r="D49" s="5" t="inlineStr">
+        <is>
+          <t>IE+UK</t>
+        </is>
+      </c>
+      <c r="E49" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F49" s="5" t="inlineStr">
+        <is>
+          <t>Exact sentence on /ie/, /uk/ "Browse by sector" and /ie/sectors/, /uk/sectors/</t>
+        </is>
+      </c>
+      <c r="G49" s="5" t="inlineStr"/>
+      <c r="H49" s="5" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>R049</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="inlineStr">
+        <is>
+          <t>Copy and credibility</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>Instead of repeatedly stating that employers say “competitive,” position: Compare disclosed salaries and identify employers committed to greater pay transparency.</t>
+        </is>
+      </c>
+      <c r="D50" s="5" t="inlineStr">
+        <is>
+          <t>IE+UK</t>
+        </is>
+      </c>
+      <c r="E50" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F50" s="5" t="inlineStr">
+        <is>
+          <t>Exact sentence on home "Salary insight", /ie/insights/, /uk/insights/ and both salary guides</t>
+        </is>
+      </c>
+      <c r="G50" s="5" t="inlineStr"/>
+      <c r="H50" s="5" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>R050</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="inlineStr">
+        <is>
+          <t>Additional improvements</t>
+        </is>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>Give the B Corp badge a short explanation</t>
+        </is>
+      </c>
+      <c r="D51" s="5" t="inlineStr">
+        <is>
+          <t>IE+UK</t>
+        </is>
+      </c>
+      <c r="E51" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F51" s="5" t="inlineStr">
+        <is>
+          <t>Hero pill (2 lines at 1440, crop ie_home_hero) + footer line + header title attribute</t>
+        </is>
+      </c>
+      <c r="G51" s="5" t="inlineStr">
+        <is>
+          <t>Wrap fixed since v1</t>
+        </is>
+      </c>
+      <c r="H51" s="5" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="7" t="inlineStr">
+        <is>
+          <t>R051</t>
+        </is>
+      </c>
+      <c r="B52" s="7" t="inlineStr">
+        <is>
+          <t>Additional improvements</t>
+        </is>
+      </c>
+      <c r="C52" s="7" t="inlineStr">
+        <is>
+          <t>Add salary guides, market reports and career advice to build repeat traffic</t>
+        </is>
+      </c>
+      <c r="D52" s="7" t="inlineStr">
+        <is>
+          <t>IE+UK</t>
+        </is>
+      </c>
+      <c r="E52" s="7" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="F52" s="7" t="inlineStr">
+        <is>
+          <t>/ie/guides/: "Green salary guide for Ireland" + 4 job-market pages; empty "Career advice and market reports" heading removed, replaced by "More guides follow as the data grows."</t>
+        </is>
+      </c>
+      <c r="G52" s="7" t="inlineStr">
+        <is>
+          <t>No career-advice or market-report content yet</t>
+        </is>
+      </c>
+      <c r="H52" s="7" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>R052</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="inlineStr">
+        <is>
+          <t>Additional improvements</t>
+        </is>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>Create dedicated SEO landing pages such as “Ecology Jobs Ireland,” “Environmental Jobs Dublin” and “Renewable Energy Jobs Ireland.”</t>
+        </is>
+      </c>
+      <c r="D53" s="5" t="inlineStr">
+        <is>
+          <t>IE+UK</t>
+        </is>
+      </c>
+      <c r="E53" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F53" s="5" t="inlineStr">
+        <is>
+          <t>/ie/ecology-jobs-ireland/, /ie/environmental-jobs-dublin/, /ie/renewable-energy-jobs-ireland/, /ie/sustainability-jobs-ireland/ + UK equivalents all 200</t>
+        </is>
+      </c>
+      <c r="G53" s="5" t="inlineStr">
+        <is>
+          <t>IE ecology page lists 2 London Mattinson roles labelled "UK" (kept per Keith rule)</t>
+        </is>
+      </c>
+      <c r="H53" s="5" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>R053</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="inlineStr">
+        <is>
+          <t>Additional improvements</t>
+        </is>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>Implement JobPosting structured data</t>
+        </is>
+      </c>
+      <c r="D54" s="5" t="inlineStr">
+        <is>
+          <t>IE+UK</t>
+        </is>
+      </c>
+      <c r="E54" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F54" s="5" t="inlineStr">
+        <is>
+          <t>&lt;script type="application/ld+json"&gt; JobPosting with Organization, Place, PostalAddress, MonetaryAmount(currency GBP on IE 11500760, EUR on UK 11501639)</t>
+        </is>
+      </c>
+      <c r="G54" s="5" t="inlineStr"/>
+      <c r="H54" s="5" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>R054</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="inlineStr">
+        <is>
+          <t>Additional improvements</t>
+        </is>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>canonical URLs</t>
+        </is>
+      </c>
+      <c r="D55" s="5" t="inlineStr">
+        <is>
+          <t>IE+UK</t>
+        </is>
+      </c>
+      <c r="E55" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F55" s="5" t="inlineStr">
+        <is>
+          <t>&lt;link rel="canonical"&gt; on every fetched page</t>
+        </is>
+      </c>
+      <c r="G55" s="5" t="inlineStr">
+        <is>
+          <t>Still points at greenjobs-redesign.pages.dev/…/index.html and every page is noindex,nofollow (demo)</t>
+        </is>
+      </c>
+      <c r="H55" s="5" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>R055</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="inlineStr">
+        <is>
+          <t>Additional improvements</t>
+        </is>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>IE/UK hreflang</t>
+        </is>
+      </c>
+      <c r="D56" s="5" t="inlineStr">
+        <is>
+          <t>IE+UK</t>
+        </is>
+      </c>
+      <c r="E56" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F56" s="5" t="inlineStr">
+        <is>
+          <t>hreflang en-IE / en-GB / x-default now on landing pages (/ie/ecology-jobs-ireland/ ↔ /uk/ecology-jobs-uk/), guides, salary guide, dashboard; job pages carry canonical only (no twin)</t>
+        </is>
+      </c>
+      <c r="G56" s="5" t="inlineStr">
+        <is>
+          <t>Landing/guide pairs added since v1</t>
+        </is>
+      </c>
+      <c r="H56" s="5" t="inlineStr">
+        <is>
+          <t>PARTIAL → DONE</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t>R056</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="inlineStr">
+        <is>
+          <t>Additional improvements</t>
+        </is>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>Test the map, animations and interactive tools for keyboard access</t>
+        </is>
+      </c>
+      <c r="D57" s="5" t="inlineStr">
+        <is>
+          <t>IE+UK</t>
+        </is>
+      </c>
+      <c r="E57" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F57" s="5" t="inlineStr">
+        <is>
+          <t>Playwright: UK map regions role=button tabindex=0 aria-label ("East Midlands: 0 roles", "Northern Ireland: 0 roles"); 404 and dialogs keyboard-closable (data-sheet-close, dialog close)</t>
+        </is>
+      </c>
+      <c r="G57" s="5" t="inlineStr"/>
+      <c r="H57" s="5" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>R057</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="inlineStr">
+        <is>
+          <t>Additional improvements</t>
+        </is>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>reduced-motion preferences</t>
+        </is>
+      </c>
+      <c r="D58" s="5" t="inlineStr">
+        <is>
+          <t>IE+UK</t>
+        </is>
+      </c>
+      <c r="E58" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F58" s="5" t="inlineStr">
+        <is>
+          <t>css/styles.css has 4 prefers-reduced-motion blocks; marquee pauses on hover/focus-within (.marq:focus-within … animation-play-state:paused)</t>
+        </is>
+      </c>
+      <c r="G58" s="5" t="inlineStr"/>
+      <c r="H58" s="5" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="7" t="inlineStr">
+        <is>
+          <t>R058</t>
+        </is>
+      </c>
+      <c r="B59" s="7" t="inlineStr">
+        <is>
+          <t>Additional improvements</t>
+        </is>
+      </c>
+      <c r="C59" s="7" t="inlineStr">
+        <is>
+          <t>mobile performance</t>
+        </is>
+      </c>
+      <c r="D59" s="7" t="inlineStr">
+        <is>
+          <t>IE+UK</t>
+        </is>
+      </c>
+      <c r="E59" s="7" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="F59" s="7" t="inlineStr">
+        <is>
+          <t>/ie/jobs/index.html 300 KB, /uk/jobs/index.html 271 KB (inline JSON); ie/data/jobs.json duplicated at 219 KB; no Lighthouse/field data</t>
+        </is>
+      </c>
+      <c r="G59" s="7" t="inlineStr">
+        <is>
+          <t>Unchanged since v1</t>
+        </is>
+      </c>
+      <c r="H59" s="7" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="8" t="inlineStr">
+        <is>
+          <t>R059</t>
+        </is>
+      </c>
+      <c r="B60" s="8" t="inlineStr">
+        <is>
+          <t>Additional improvements</t>
+        </is>
+      </c>
+      <c r="C60" s="8" t="inlineStr">
+        <is>
+          <t>Replace “3 employers” with employer logos only if each relationship and permission to display the logo are current.</t>
+        </is>
+      </c>
+      <c r="D60" s="8" t="inlineStr">
+        <is>
+          <t>IE+UK</t>
+        </is>
+      </c>
+      <c r="E60" s="8" t="inlineStr">
+        <is>
+          <t>NEEDS CLIENT INPUT</t>
+        </is>
+      </c>
+      <c r="F60" s="8" t="inlineStr">
+        <is>
+          <t>IE strip shows only the 3 organisations with live roles (Mattinson logo, Commonland/Gaia text); UK strip 12 logos from listings</t>
+        </is>
+      </c>
+      <c r="G60" s="8" t="inlineStr">
+        <is>
+          <t>Text tiles for Commonland/Gaia; permissions still to be confirmed by client</t>
+        </is>
+      </c>
+      <c r="H60" s="8" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="5" t="inlineStr">
+        <is>
+          <t>R060</t>
+        </is>
+      </c>
+      <c r="B61" s="5" t="inlineStr">
+        <is>
+          <t>UK: geography</t>
+        </is>
+      </c>
+      <c r="C61" s="5" t="inlineStr">
+        <is>
+          <t>The UK homepage currently contains too much Irish inventory / tighter geographic separation</t>
+        </is>
+      </c>
+      <c r="D61" s="5" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="E61" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F61" s="5" t="inlineStr">
+        <is>
+          <t>uk/data/jobs.json: 77 = 74 uk + 3 cross; 0 ie-only</t>
+        </is>
+      </c>
+      <c r="G61" s="5" t="inlineStr"/>
+      <c r="H61" s="5" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="5" t="inlineStr">
+        <is>
+          <t>R061</t>
+        </is>
+      </c>
+      <c r="B62" s="5" t="inlineStr">
+        <is>
+          <t>UK: geography</t>
+        </is>
+      </c>
+      <c r="C62" s="5" t="inlineStr">
+        <is>
+          <t>Keep Irish-only vacancies off the UK homepage — Two Dublin-only Gaia roles appear in the latest UK vacancies.</t>
+        </is>
+      </c>
+      <c r="D62" s="5" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="E62" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F62" s="5" t="inlineStr">
+        <is>
+          <t>/uk/ Latest UK roles: 8 cards, none Dublin-only; Gaia role shown as "Dublin, United Kingdom (UK) · Ireland &amp; UK"</t>
+        </is>
+      </c>
+      <c r="G62" s="5" t="inlineStr"/>
+      <c r="H62" s="5" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="5" t="inlineStr">
+        <is>
+          <t>R062</t>
+        </is>
+      </c>
+      <c r="B63" s="5" t="inlineStr">
+        <is>
+          <t>UK: geography</t>
+        </is>
+      </c>
+      <c r="C63" s="5" t="inlineStr">
+        <is>
+          <t>23 of the 98 roles are classified as “Ireland &amp; abroad.”</t>
+        </is>
+      </c>
+      <c r="D63" s="5" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="E63" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F63" s="5" t="inlineStr">
+        <is>
+          <t>No "Ireland &amp; abroad" bucket (grep 0); headline 77; "13 roles are not on the map: UK-wide / remote (13)"</t>
+        </is>
+      </c>
+      <c r="G63" s="5" t="inlineStr"/>
+      <c r="H63" s="5" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="5" t="inlineStr">
+        <is>
+          <t>R063</t>
+        </is>
+      </c>
+      <c r="B64" s="5" t="inlineStr">
+        <is>
+          <t>UK: geography</t>
+        </is>
+      </c>
+      <c r="C64" s="5" t="inlineStr">
+        <is>
+          <t>Only show a vacancy on the UK edition where it is: Located in the UK</t>
+        </is>
+      </c>
+      <c r="D64" s="5" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="E64" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F64" s="5" t="inlineStr">
+        <is>
+          <t>uk jobs.json loc_class: 74 uk</t>
+        </is>
+      </c>
+      <c r="G64" s="5" t="inlineStr"/>
+      <c r="H64" s="5" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="5" t="inlineStr">
+        <is>
+          <t>R064</t>
+        </is>
+      </c>
+      <c r="B65" s="5" t="inlineStr">
+        <is>
+          <t>UK: geography</t>
+        </is>
+      </c>
+      <c r="C65" s="5" t="inlineStr">
+        <is>
+          <t>Fully remote and open to UK residents</t>
+        </is>
+      </c>
+      <c r="D65" s="5" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="E65" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F65" s="5" t="inlineStr">
+        <is>
+          <t>7 remote-workplace roles in UK dataset; Workplace filter has Remote</t>
+        </is>
+      </c>
+      <c r="G65" s="5" t="inlineStr"/>
+      <c r="H65" s="5" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="5" t="inlineStr">
+        <is>
+          <t>R065</t>
+        </is>
+      </c>
+      <c r="B66" s="5" t="inlineStr">
+        <is>
+          <t>UK: geography</t>
+        </is>
+      </c>
+      <c r="C66" s="5" t="inlineStr">
+        <is>
+          <t>Explicitly available in both the UK and Ireland</t>
+        </is>
+      </c>
+      <c r="D66" s="5" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="E66" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F66" s="5" t="inlineStr">
+        <is>
+          <t>3 "cross" roles labelled "Ireland &amp; UK"</t>
+        </is>
+      </c>
+      <c r="G66" s="5" t="inlineStr"/>
+      <c r="H66" s="5" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="5" t="inlineStr">
+        <is>
+          <t>R066</t>
+        </is>
+      </c>
+      <c r="B67" s="5" t="inlineStr">
+        <is>
+          <t>UK: geography</t>
+        </is>
+      </c>
+      <c r="C67" s="5" t="inlineStr">
+        <is>
+          <t>The headline should reflect genuine UK availability, not the entire shared database.</t>
+        </is>
+      </c>
+      <c r="D67" s="5" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="E67" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F67" s="5" t="inlineStr">
+        <is>
+          <t>/uk/ "77 live green roles across the UK this week"</t>
+        </is>
+      </c>
+      <c r="G67" s="5" t="inlineStr"/>
+      <c r="H67" s="5" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="5" t="inlineStr">
+        <is>
+          <t>R067</t>
+        </is>
+      </c>
+      <c r="B68" s="5" t="inlineStr">
+        <is>
+          <t>UK: geography</t>
+        </is>
+      </c>
+      <c r="C68" s="5" t="inlineStr">
+        <is>
+          <t>Do not show euro salaries without explanation — The Commonland role displays €5.1k–€6k/month on the UK homepage.</t>
+        </is>
+      </c>
+      <c r="D68" s="5" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="E68" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F68" s="5" t="inlineStr">
+        <is>
+          <t>/uk/ card: "€5.1k–6k/mo" chip + separate "paid in € ≈ £4.4k–5.1k/mo" chip (crop uk_home_marquee_after3s)</t>
+        </is>
+      </c>
+      <c r="G68" s="5" t="inlineStr">
+        <is>
+          <t>Long chip split in two since v1; no mid-value wrap at 390 (crop uk_home390_mid)</t>
+        </is>
+      </c>
+      <c r="H68" s="5" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="5" t="inlineStr">
+        <is>
+          <t>R068</t>
+        </is>
+      </c>
+      <c r="B69" s="5" t="inlineStr">
+        <is>
+          <t>UK: geography</t>
+        </is>
+      </c>
+      <c r="C69" s="5" t="inlineStr">
+        <is>
+          <t>Show the original salary with a clear “salary paid in euros” label</t>
+        </is>
+      </c>
+      <c r="D69" s="5" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="E69" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F69" s="5" t="inlineStr">
+        <is>
+          <t>"(paid in euros, about £4.4k–5.1k/mo)" on the job page; "paid in €" chip on cards</t>
+        </is>
+      </c>
+      <c r="G69" s="5" t="inlineStr"/>
+      <c r="H69" s="5" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="5" t="inlineStr">
+        <is>
+          <t>R069</t>
+        </is>
+      </c>
+      <c r="B70" s="5" t="inlineStr">
+        <is>
+          <t>UK: geography</t>
+        </is>
+      </c>
+      <c r="C70" s="5" t="inlineStr">
+        <is>
+          <t>Provide an approximate sterling equivalent alongside it.</t>
+        </is>
+      </c>
+      <c r="D70" s="5" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="E70" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F70" s="5" t="inlineStr">
+        <is>
+          <t>"about £4.4k–5.1k/mo"</t>
+        </is>
+      </c>
+      <c r="G70" s="5" t="inlineStr"/>
+      <c r="H70" s="5" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="5" t="inlineStr">
+        <is>
+          <t>R070</t>
+        </is>
+      </c>
+      <c r="B71" s="5" t="inlineStr">
+        <is>
+          <t>UK: geography</t>
+        </is>
+      </c>
+      <c r="C71" s="5" t="inlineStr">
+        <is>
+          <t>Do not silently convert salaries for UK vacancies.</t>
+        </is>
+      </c>
+      <c r="D71" s="5" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="E71" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F71" s="5" t="inlineStr">
+        <is>
+          <t>UK dataset: 46 GBP, 1 EUR (labelled), 30 undisclosed</t>
+        </is>
+      </c>
+      <c r="G71" s="5" t="inlineStr"/>
+      <c r="H71" s="5" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="5" t="inlineStr">
+        <is>
+          <t>R071</t>
+        </is>
+      </c>
+      <c r="B72" s="5" t="inlineStr">
+        <is>
+          <t>UK: geography</t>
+        </is>
+      </c>
+      <c r="C72" s="5" t="inlineStr">
+        <is>
+          <t>“Every region, counted” is slightly misleading</t>
+        </is>
+      </c>
+      <c r="D72" s="5" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="E72" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F72" s="5" t="inlineStr">
+        <is>
+          <t>"Every region, counted" only in for-keith quote; section h2 "See where green employers are hiring"</t>
+        </is>
+      </c>
+      <c r="G72" s="5" t="inlineStr"/>
+      <c r="H72" s="5" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="7" t="inlineStr">
+        <is>
+          <t>R072</t>
+        </is>
+      </c>
+      <c r="B73" s="7" t="inlineStr">
+        <is>
+          <t>UK: geography</t>
+        </is>
+      </c>
+      <c r="C73" s="7" t="inlineStr">
+        <is>
+          <t>Northern Ireland is absent.</t>
+        </is>
+      </c>
+      <c r="D73" s="7" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="E73" s="7" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="F73" s="7" t="inlineStr">
+        <is>
+          <t>Map has a Northern Ireland region (aria "Northern Ireland: 0 roles"); region list now includes "Northern Ireland 0" and the datalist has an "Northern Ireland" option (uk/jobs/index.html)</t>
+        </is>
+      </c>
+      <c r="G73" s="7" t="inlineStr">
+        <is>
+          <t>Improved: NI is a filter option now. NI still renders as a dark hole on the map (crop uk_home_map) — see visual #12</t>
+        </is>
+      </c>
+      <c r="H73" s="7" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="5" t="inlineStr">
+        <is>
+          <t>R073</t>
+        </is>
+      </c>
+      <c r="B74" s="5" t="inlineStr">
+        <is>
+          <t>UK: geography</t>
+        </is>
+      </c>
+      <c r="C74" s="5" t="inlineStr">
+        <is>
+          <t>East Midlands is absent.</t>
+        </is>
+      </c>
+      <c r="D74" s="5" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="E74" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F74" s="5" t="inlineStr">
+        <is>
+          <t>Region list shows "East Midlands 0"; map region aria "East Midlands: 0 roles"</t>
+        </is>
+      </c>
+      <c r="G74" s="5" t="inlineStr">
+        <is>
+          <t>Listed at 0 since v1</t>
+        </is>
+      </c>
+      <c r="H74" s="5" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="5" t="inlineStr">
+        <is>
+          <t>R074</t>
+        </is>
+      </c>
+      <c r="B75" s="5" t="inlineStr">
+        <is>
+          <t>UK: geography</t>
+        </is>
+      </c>
+      <c r="C75" s="5" t="inlineStr">
+        <is>
+          <t>Ireland and overseas roles are grouped separately.</t>
+        </is>
+      </c>
+      <c r="D75" s="5" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="E75" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F75" s="5" t="inlineStr">
+        <is>
+          <t>Only "UK-wide / remote (13)" as the off-map group</t>
+        </is>
+      </c>
+      <c r="G75" s="5" t="inlineStr"/>
+      <c r="H75" s="5" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="5" t="inlineStr">
+        <is>
+          <t>R075</t>
+        </is>
+      </c>
+      <c r="B76" s="5" t="inlineStr">
+        <is>
+          <t>UK: geography</t>
+        </is>
+      </c>
+      <c r="C76" s="5" t="inlineStr">
+        <is>
+          <t>UK-wide roles are not shown on the map.</t>
+        </is>
+      </c>
+      <c r="D76" s="5" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="E76" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F76" s="5" t="inlineStr">
+        <is>
+          <t>"13 roles are not on the map: UK-wide / remote (13)" link beside the map</t>
+        </is>
+      </c>
+      <c r="G76" s="5" t="inlineStr"/>
+      <c r="H76" s="5" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="5" t="inlineStr">
+        <is>
+          <t>R076</t>
+        </is>
+      </c>
+      <c r="B77" s="5" t="inlineStr">
+        <is>
+          <t>UK: geography</t>
+        </is>
+      </c>
+      <c r="C77" s="5" t="inlineStr">
+        <is>
+          <t>A better heading would be: See where green employers are hiring — Explore current vacancies by UK region, including nationwide and remote opportunities.</t>
+        </is>
+      </c>
+      <c r="D77" s="5" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="E77" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F77" s="5" t="inlineStr">
+        <is>
+          <t>/uk/ h2 + lede are the exact sentences</t>
+        </is>
+      </c>
+      <c r="G77" s="5" t="inlineStr"/>
+      <c r="H77" s="5" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="5" t="inlineStr">
+        <is>
+          <t>R077</t>
+        </is>
+      </c>
+      <c r="B78" s="5" t="inlineStr">
+        <is>
+          <t>UK: geography</t>
+        </is>
+      </c>
+      <c r="C78" s="5" t="inlineStr">
+        <is>
+          <t>Northern Ireland should be included as a clear location option</t>
+        </is>
+      </c>
+      <c r="D78" s="5" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="E78" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F78" s="5" t="inlineStr">
+        <is>
+          <t>"Northern Ireland" appears in the region list (0) and in the /uk/jobs/ region datalist (grep count 5)</t>
+        </is>
+      </c>
+      <c r="G78" s="5" t="inlineStr">
+        <is>
+          <t>Was PARTIAL; option added since v1</t>
+        </is>
+      </c>
+      <c r="H78" s="5" t="inlineStr">
+        <is>
+          <t>PARTIAL → DONE</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="5" t="inlineStr">
+        <is>
+          <t>R078</t>
+        </is>
+      </c>
+      <c r="B79" s="5" t="inlineStr">
+        <is>
+          <t>UK: matching examples</t>
+        </is>
+      </c>
+      <c r="C79" s="5" t="inlineStr">
+        <is>
+          <t>Remove Dublin from the matching example (ecologist dublin)</t>
+        </is>
+      </c>
+      <c r="D79" s="5" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="E79" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F79" s="5" t="inlineStr">
+        <is>
+          <t>/uk/jobs/ examples: no Dublin; placeholder ends "…EIA chapters, Bristol"</t>
+        </is>
+      </c>
+      <c r="G79" s="5" t="inlineStr"/>
+      <c r="H79" s="5" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="5" t="inlineStr">
+        <is>
+          <t>R079</t>
+        </is>
+      </c>
+      <c r="B80" s="5" t="inlineStr">
+        <is>
+          <t>UK: matching examples</t>
+        </is>
+      </c>
+      <c r="C80" s="5" t="inlineStr">
+        <is>
+          <t>ecologist Bristol</t>
+        </is>
+      </c>
+      <c r="D80" s="5" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="E80" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F80" s="5" t="inlineStr">
+        <is>
+          <t>"Try:" chip "ecologist Bristol"</t>
+        </is>
+      </c>
+      <c r="G80" s="5" t="inlineStr"/>
+      <c r="H80" s="5" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="5" t="inlineStr">
+        <is>
+          <t>R080</t>
+        </is>
+      </c>
+      <c r="B81" s="5" t="inlineStr">
+        <is>
+          <t>UK: matching examples</t>
+        </is>
+      </c>
+      <c r="C81" s="5" t="inlineStr">
+        <is>
+          <t>sustainability consultant London</t>
+        </is>
+      </c>
+      <c r="D81" s="5" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="E81" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F81" s="5" t="inlineStr">
+        <is>
+          <t>chip "sustainability consultant London"</t>
+        </is>
+      </c>
+      <c r="G81" s="5" t="inlineStr"/>
+      <c r="H81" s="5" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="5" t="inlineStr">
+        <is>
+          <t>R081</t>
+        </is>
+      </c>
+      <c r="B82" s="5" t="inlineStr">
+        <is>
+          <t>UK: matching examples</t>
+        </is>
+      </c>
+      <c r="C82" s="5" t="inlineStr">
+        <is>
+          <t>flood risk engineer Manchester</t>
+        </is>
+      </c>
+      <c r="D82" s="5" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="E82" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F82" s="5" t="inlineStr">
+        <is>
+          <t>chip "flood risk engineer Manchester"</t>
+        </is>
+      </c>
+      <c r="G82" s="5" t="inlineStr"/>
+      <c r="H82" s="5" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="5" t="inlineStr">
+        <is>
+          <t>R082</t>
+        </is>
+      </c>
+      <c r="B83" s="5" t="inlineStr">
+        <is>
+          <t>UK: matching examples</t>
+        </is>
+      </c>
+      <c r="C83" s="5" t="inlineStr">
+        <is>
+          <t>renewable energy Scotland</t>
+        </is>
+      </c>
+      <c r="D83" s="5" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="E83" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F83" s="5" t="inlineStr">
+        <is>
+          <t>chip "renewable energy Scotland"</t>
+        </is>
+      </c>
+      <c r="G83" s="5" t="inlineStr"/>
+      <c r="H83" s="5" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="5" t="inlineStr">
+        <is>
+          <t>R083</t>
+        </is>
+      </c>
+      <c r="B84" s="5" t="inlineStr">
+        <is>
+          <t>UK: contact</t>
+        </is>
+      </c>
+      <c r="C84" s="5" t="inlineStr">
+        <is>
+          <t>Correct the UK contact information — footer says “Calling From Ireland” / “Calling From Outside Ireland”</t>
+        </is>
+      </c>
+      <c r="D84" s="5" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="E84" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F84" s="5" t="inlineStr">
+        <is>
+          <t>"Calling From Outside" only in for-keith quote</t>
+        </is>
+      </c>
+      <c r="G84" s="5" t="inlineStr"/>
+      <c r="H84" s="5" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="5" t="inlineStr">
+        <is>
+          <t>R084</t>
+        </is>
+      </c>
+      <c r="B85" s="5" t="inlineStr">
+        <is>
+          <t>UK: contact</t>
+        </is>
+      </c>
+      <c r="C85" s="5" t="inlineStr">
+        <is>
+          <t>Calling from the UK: +44 28 4303 2055</t>
+        </is>
+      </c>
+      <c r="D85" s="5" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="E85" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F85" s="5" t="inlineStr">
+        <is>
+          <t>/uk/ footer first line "Calling from the UK: +44 28 4303 2055"</t>
+        </is>
+      </c>
+      <c r="G85" s="5" t="inlineStr"/>
+      <c r="H85" s="5" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="5" t="inlineStr">
+        <is>
+          <t>R085</t>
+        </is>
+      </c>
+      <c r="B86" s="5" t="inlineStr">
+        <is>
+          <t>UK: contact</t>
+        </is>
+      </c>
+      <c r="C86" s="5" t="inlineStr">
+        <is>
+          <t>Calling from Ireland: (01) 912 5247</t>
+        </is>
+      </c>
+      <c r="D86" s="5" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="E86" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F86" s="5" t="inlineStr">
+        <is>
+          <t>/uk/ footer second line "Calling from Ireland: (01) 912 5247"; IE footer lists Ireland first</t>
+        </is>
+      </c>
+      <c r="G86" s="5" t="inlineStr"/>
+      <c r="H86" s="5" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="8" t="inlineStr">
+        <is>
+          <t>R086</t>
+        </is>
+      </c>
+      <c r="B87" s="8" t="inlineStr">
+        <is>
+          <t>UK: contact</t>
+        </is>
+      </c>
+      <c r="C87" s="8" t="inlineStr">
+        <is>
+          <t>A GB number could also help. A Northern Ireland number may make some English employers assume the business primarily covers Ireland.</t>
+        </is>
+      </c>
+      <c r="D87" s="8" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="E87" s="8" t="inlineStr">
+        <is>
+          <t>NEEDS CLIENT INPUT</t>
+        </is>
+      </c>
+      <c r="F87" s="8" t="inlineStr">
+        <is>
+          <t>Only +44 28 (NI) number on /uk/</t>
+        </is>
+      </c>
+      <c r="G87" s="8" t="inlineStr">
+        <is>
+          <t>Client must provide a GB number</t>
+        </is>
+      </c>
+      <c r="H87" s="8" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="5" t="inlineStr">
+        <is>
+          <t>R087</t>
+        </is>
+      </c>
+      <c r="B88" s="5" t="inlineStr">
+        <is>
+          <t>UK: sector classification</t>
+        </is>
+      </c>
+      <c r="C88" s="5" t="inlineStr">
+        <is>
+          <t>Highways Civil Engineer appears under “Built environment &amp; energy efficiency.” Should be under infrastructure, transportation or civil engineering.</t>
+        </is>
+      </c>
+      <c r="D88" s="5" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="E88" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F88" s="5" t="inlineStr">
+        <is>
+          <t>/uk/jobs/11501402/ Sector row = "Sustainable infrastructure &amp; transport" only; jobs.json sectors ["Sustainable infrastructure &amp; transport"]</t>
+        </is>
+      </c>
+      <c r="G88" s="5" t="inlineStr">
+        <is>
+          <t>Built-environment tag dropped since v1</t>
+        </is>
+      </c>
+      <c r="H88" s="5" t="inlineStr">
+        <is>
+          <t>PARTIAL → DONE</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="5" t="inlineStr">
+        <is>
+          <t>R088</t>
+        </is>
+      </c>
+      <c r="B89" s="5" t="inlineStr">
+        <is>
+          <t>UK: sector classification</t>
+        </is>
+      </c>
+      <c r="C89" s="5" t="inlineStr">
+        <is>
+          <t>I would consider adding: Environmental engineering</t>
+        </is>
+      </c>
+      <c r="D89" s="5" t="inlineStr">
+        <is>
+          <t>IE+UK</t>
+        </is>
+      </c>
+      <c r="E89" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F89" s="5" t="inlineStr">
+        <is>
+          <t>IE "Environmental engineering" (8 roles); UK 0 roles so hidden ("No empty categories")</t>
+        </is>
+      </c>
+      <c r="G89" s="5" t="inlineStr"/>
+      <c r="H89" s="5" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="5" t="inlineStr">
+        <is>
+          <t>R089</t>
+        </is>
+      </c>
+      <c r="B90" s="5" t="inlineStr">
+        <is>
+          <t>UK: sector classification</t>
+        </is>
+      </c>
+      <c r="C90" s="5" t="inlineStr">
+        <is>
+          <t>Sustainable infrastructure</t>
+        </is>
+      </c>
+      <c r="D90" s="5" t="inlineStr">
+        <is>
+          <t>IE+UK</t>
+        </is>
+      </c>
+      <c r="E90" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F90" s="5" t="inlineStr">
+        <is>
+          <t>"Sustainable infrastructure &amp; transport" (IE 33 / UK 18)</t>
+        </is>
+      </c>
+      <c r="G90" s="5" t="inlineStr"/>
+      <c r="H90" s="5" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="6" t="inlineStr">
+        <is>
+          <t>R090</t>
+        </is>
+      </c>
+      <c r="B91" s="6" t="inlineStr">
+        <is>
+          <t>UK: sector classification</t>
+        </is>
+      </c>
+      <c r="C91" s="6" t="inlineStr">
+        <is>
+          <t>Transport and active travel</t>
+        </is>
+      </c>
+      <c r="D91" s="6" t="inlineStr">
+        <is>
+          <t>IE+UK</t>
+        </is>
+      </c>
+      <c r="E91" s="6" t="inlineStr">
+        <is>
+          <t>INTERPRETED DIFFERENTLY</t>
+        </is>
+      </c>
+      <c r="F91" s="6" t="inlineStr">
+        <is>
+          <t>Merged into "Sustainable infrastructure &amp; transport"; no standalone transport/active-travel sector</t>
+        </is>
+      </c>
+      <c r="G91" s="6" t="inlineStr">
+        <is>
+          <t>Client to confirm the merge</t>
+        </is>
+      </c>
+      <c r="H91" s="6" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="5" t="inlineStr">
+        <is>
+          <t>R091</t>
+        </is>
+      </c>
+      <c r="B92" s="5" t="inlineStr">
+        <is>
+          <t>UK: sector classification</t>
+        </is>
+      </c>
+      <c r="C92" s="5" t="inlineStr">
+        <is>
+          <t>Climate and carbon</t>
+        </is>
+      </c>
+      <c r="D92" s="5" t="inlineStr">
+        <is>
+          <t>IE+UK</t>
+        </is>
+      </c>
+      <c r="E92" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F92" s="5" t="inlineStr">
+        <is>
+          <t>"Climate &amp; carbon" (IE 1 / UK 5)</t>
+        </is>
+      </c>
+      <c r="G92" s="5" t="inlineStr"/>
+      <c r="H92" s="5" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="5" t="inlineStr">
+        <is>
+          <t>R092</t>
+        </is>
+      </c>
+      <c r="B93" s="5" t="inlineStr">
+        <is>
+          <t>UK: sector classification</t>
+        </is>
+      </c>
+      <c r="C93" s="5" t="inlineStr">
+        <is>
+          <t>Health, safety and environmental</t>
+        </is>
+      </c>
+      <c r="D93" s="5" t="inlineStr">
+        <is>
+          <t>IE+UK</t>
+        </is>
+      </c>
+      <c r="E93" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F93" s="5" t="inlineStr">
+        <is>
+          <t>"Health, safety &amp; environment" (IE 11 / UK 8)</t>
+        </is>
+      </c>
+      <c r="G93" s="5" t="inlineStr"/>
+      <c r="H93" s="5" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="5" t="inlineStr">
+        <is>
+          <t>R093</t>
+        </is>
+      </c>
+      <c r="B94" s="5" t="inlineStr">
+        <is>
+          <t>UK: sector classification</t>
+        </is>
+      </c>
+      <c r="C94" s="5" t="inlineStr">
+        <is>
+          <t>Nature recovery and biodiversity</t>
+        </is>
+      </c>
+      <c r="D94" s="5" t="inlineStr">
+        <is>
+          <t>IE+UK</t>
+        </is>
+      </c>
+      <c r="E94" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F94" s="5" t="inlineStr">
+        <is>
+          <t>"Ecology, nature recovery &amp; biodiversity" (IE 10 / UK 17)</t>
+        </is>
+      </c>
+      <c r="G94" s="5" t="inlineStr"/>
+      <c r="H94" s="5" t="inlineStr"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="5" t="inlineStr">
+        <is>
+          <t>R094</t>
+        </is>
+      </c>
+      <c r="B95" s="5" t="inlineStr">
+        <is>
+          <t>UK: sector classification</t>
+        </is>
+      </c>
+      <c r="C95" s="5" t="inlineStr">
+        <is>
+          <t>The categorisation must be consistent because the salary explorer and sector statistics depend on it.</t>
+        </is>
+      </c>
+      <c r="D95" s="5" t="inlineStr">
+        <is>
+          <t>IE+UK</t>
+        </is>
+      </c>
+      <c r="E95" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F95" s="5" t="inlineStr">
+        <is>
+          <t>Same 14-name taxonomy on jobs filter, sectors page, salary explorer, salary guide, dashboard and alert form (text dumps)</t>
+        </is>
+      </c>
+      <c r="G95" s="5" t="inlineStr"/>
+      <c r="H95" s="5" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="8" t="inlineStr">
+        <is>
+          <t>R095</t>
+        </is>
+      </c>
+      <c r="B96" s="8" t="inlineStr">
+        <is>
+          <t>UK: credibility signals</t>
+        </is>
+      </c>
+      <c r="C96" s="8" t="inlineStr">
+        <is>
+          <t>UK employer testimonials</t>
+        </is>
+      </c>
+      <c r="D96" s="8" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="E96" s="8" t="inlineStr">
+        <is>
+          <t>NEEDS CLIENT INPUT</t>
+        </is>
+      </c>
+      <c r="F96" s="8" t="inlineStr">
+        <is>
+          <t>/uk/employers/ "Trusted across the UK — Client testimonials are being collected for launch."</t>
+        </is>
+      </c>
+      <c r="G96" s="8" t="inlineStr">
+        <is>
+          <t>Client must supply quotes</t>
+        </is>
+      </c>
+      <c r="H96" s="8" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="5" t="inlineStr">
+        <is>
+          <t>R096</t>
+        </is>
+      </c>
+      <c r="B97" s="5" t="inlineStr">
+        <is>
+          <t>UK: credibility signals</t>
+        </is>
+      </c>
+      <c r="C97" s="5" t="inlineStr">
+        <is>
+          <t>Recognisable organisations that have recruited through the network</t>
+        </is>
+      </c>
+      <c r="D97" s="5" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="E97" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F97" s="5" t="inlineStr">
+        <is>
+          <t>/uk/employers/ + /uk/ marquee: Arup, Commonland, Dacorum BC, Environmental Standards Scotland, Gaia Talent, Grundon, Haskoning, Jacobs, … (12 logos)</t>
+        </is>
+      </c>
+      <c r="G97" s="5" t="inlineStr"/>
+      <c r="H97" s="5" t="inlineStr"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="8" t="inlineStr">
+        <is>
+          <t>R097</t>
+        </is>
+      </c>
+      <c r="B98" s="8" t="inlineStr">
+        <is>
+          <t>UK: credibility signals</t>
+        </is>
+      </c>
+      <c r="C98" s="8" t="inlineStr">
+        <is>
+          <t>Candidate and email audience figures</t>
+        </is>
+      </c>
+      <c r="D98" s="8" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="E98" s="8" t="inlineStr">
+        <is>
+          <t>NEEDS CLIENT INPUT</t>
+        </is>
+      </c>
+      <c r="F98" s="8" t="inlineStr">
+        <is>
+          <t>"Monthly visitor figures are published at launch." / "Subscriber numbers are published at launch."</t>
+        </is>
+      </c>
+      <c r="G98" s="8" t="inlineStr"/>
+      <c r="H98" s="8" t="inlineStr"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="8" t="inlineStr">
+        <is>
+          <t>R098</t>
+        </is>
+      </c>
+      <c r="B99" s="8" t="inlineStr">
+        <is>
+          <t>UK: credibility signals</t>
+        </is>
+      </c>
+      <c r="C99" s="8" t="inlineStr">
+        <is>
+          <t>LinkedIn distribution</t>
+        </is>
+      </c>
+      <c r="D99" s="8" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="E99" s="8" t="inlineStr">
+        <is>
+          <t>NEEDS CLIENT INPUT</t>
+        </is>
+      </c>
+      <c r="F99" s="8" t="inlineStr">
+        <is>
+          <t>"Network and follower numbers are published at launch."</t>
+        </is>
+      </c>
+      <c r="G99" s="8" t="inlineStr"/>
+      <c r="H99" s="8" t="inlineStr"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="9" t="inlineStr">
+        <is>
+          <t>R099</t>
+        </is>
+      </c>
+      <c r="B100" s="9" t="inlineStr">
+        <is>
+          <t>UK: credibility signals</t>
+        </is>
+      </c>
+      <c r="C100" s="9" t="inlineStr">
+        <is>
+          <t>Examples of UK placements or campaigns</t>
+        </is>
+      </c>
+      <c r="D100" s="9" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="E100" s="9" t="inlineStr">
+        <is>
+          <t>NOT DONE</t>
+        </is>
+      </c>
+      <c r="F100" s="9" t="inlineStr">
+        <is>
+          <t>No placement or campaign example on /uk/employers/ or /uk/ (grep "placement", "campaign": 0)</t>
+        </is>
+      </c>
+      <c r="G100" s="9" t="inlineStr">
+        <is>
+          <t>Unchanged; needs client case material</t>
+        </is>
+      </c>
+      <c r="H100" s="9" t="inlineStr"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="5" t="inlineStr">
+        <is>
+          <t>R100</t>
+        </is>
+      </c>
+      <c r="B101" s="5" t="inlineStr">
+        <is>
+          <t>UK: credibility signals</t>
+        </is>
+      </c>
+      <c r="C101" s="5" t="inlineStr">
+        <is>
+          <t>Coverage across the ten-site specialist network</t>
+        </is>
+      </c>
+      <c r="D101" s="5" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="E101" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F101" s="5" t="inlineStr">
+        <is>
+          <t>/uk/employers/ "Network coverage: conservationjobsuk.com … windjobsuk.com" (10) and "The network" chips on home</t>
+        </is>
+      </c>
+      <c r="G101" s="5" t="inlineStr"/>
+      <c r="H101" s="5" t="inlineStr"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="5" t="inlineStr">
+        <is>
+          <t>R101</t>
+        </is>
+      </c>
+      <c r="B102" s="5" t="inlineStr">
+        <is>
+          <t>UK: credibility signals</t>
+        </is>
+      </c>
+      <c r="C102" s="5" t="inlineStr">
+        <is>
+          <t>A clear UK advertising price or rate-card CTA</t>
+        </is>
+      </c>
+      <c r="D102" s="5" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="E102" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F102" s="5" t="inlineStr">
+        <is>
+          <t>"Request advertising rates →" ×3 on /uk/employers/</t>
+        </is>
+      </c>
+      <c r="G102" s="5" t="inlineStr"/>
+      <c r="H102" s="5" t="inlineStr"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="5" t="inlineStr">
+        <is>
+          <t>R102</t>
+        </is>
+      </c>
+      <c r="B103" s="5" t="inlineStr">
+        <is>
+          <t>UK: credibility signals</t>
+        </is>
+      </c>
+      <c r="C103" s="5" t="inlineStr">
+        <is>
+          <t>The statement “19 employers hiring now” is worth retaining on the UK site.</t>
+        </is>
+      </c>
+      <c r="D103" s="5" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="E103" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F103" s="5" t="inlineStr">
+        <is>
+          <t>/uk/ hero strip "18 employers hiring now" (live count)</t>
+        </is>
+      </c>
+      <c r="G103" s="5" t="inlineStr"/>
+      <c r="H103" s="5" t="inlineStr"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="5" t="inlineStr">
+        <is>
+          <t>R103</t>
+        </is>
+      </c>
+      <c r="B104" s="5" t="inlineStr">
+        <is>
+          <t>UK: proposition</t>
+        </is>
+      </c>
+      <c r="C104" s="5" t="inlineStr">
+        <is>
+          <t>Add a plain-English subheading beneath the tagline: Search environmental, ecology, sustainability, renewable-energy and low-carbon careers across the UK.</t>
+        </is>
+      </c>
+      <c r="D104" s="5" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="E104" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F104" s="5" t="inlineStr">
+        <is>
+          <t>/uk/ hero subheading is the exact sentence</t>
+        </is>
+      </c>
+      <c r="G104" s="5" t="inlineStr"/>
+      <c r="H104" s="5" t="inlineStr"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="5" t="inlineStr">
+        <is>
+          <t>R104</t>
+        </is>
+      </c>
+      <c r="B105" s="5" t="inlineStr">
+        <is>
+          <t>UK: homepage order</t>
+        </is>
+      </c>
+      <c r="C105" s="5" t="inlineStr">
+        <is>
+          <t>Reduce homepage repetition — Regions, sectors and salary information each appear more than once.</t>
+        </is>
+      </c>
+      <c r="D105" s="5" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="E105" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F105" s="5" t="inlineStr">
+        <is>
+          <t>/uk/: one region section, one sector section, one salary section</t>
+        </is>
+      </c>
+      <c r="G105" s="5" t="inlineStr"/>
+      <c r="H105" s="5" t="inlineStr"/>
+    </row>
+    <row r="106">
+      <c r="A106" s="5" t="inlineStr">
+        <is>
+          <t>R105</t>
+        </is>
+      </c>
+      <c r="B106" s="5" t="inlineStr">
+        <is>
+          <t>UK: homepage order</t>
+        </is>
+      </c>
+      <c r="C106" s="5" t="inlineStr">
+        <is>
+          <t>Search and headline</t>
+        </is>
+      </c>
+      <c r="D106" s="5" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="E106" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F106" s="5" t="inlineStr">
+        <is>
+          <t>/uk/ hero with search first</t>
+        </is>
+      </c>
+      <c r="G106" s="5" t="inlineStr"/>
+      <c r="H106" s="5" t="inlineStr"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="5" t="inlineStr">
+        <is>
+          <t>R106</t>
+        </is>
+      </c>
+      <c r="B107" s="5" t="inlineStr">
+        <is>
+          <t>UK: homepage order</t>
+        </is>
+      </c>
+      <c r="C107" s="5" t="inlineStr">
+        <is>
+          <t>Latest UK roles</t>
+        </is>
+      </c>
+      <c r="D107" s="5" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="E107" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F107" s="5" t="inlineStr">
+        <is>
+          <t>"Latest UK roles" second</t>
+        </is>
+      </c>
+      <c r="G107" s="5" t="inlineStr"/>
+      <c r="H107" s="5" t="inlineStr"/>
+    </row>
+    <row r="108">
+      <c r="A108" s="5" t="inlineStr">
+        <is>
+          <t>R107</t>
+        </is>
+      </c>
+      <c r="B108" s="5" t="inlineStr">
+        <is>
+          <t>UK: homepage order</t>
+        </is>
+      </c>
+      <c r="C108" s="5" t="inlineStr">
+        <is>
+          <t>Browse by sector</t>
+        </is>
+      </c>
+      <c r="D108" s="5" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="E108" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F108" s="5" t="inlineStr">
+        <is>
+          <t>"Browse by sector" third</t>
+        </is>
+      </c>
+      <c r="G108" s="5" t="inlineStr"/>
+      <c r="H108" s="5" t="inlineStr"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="5" t="inlineStr">
+        <is>
+          <t>R108</t>
+        </is>
+      </c>
+      <c r="B109" s="5" t="inlineStr">
+        <is>
+          <t>UK: homepage order</t>
+        </is>
+      </c>
+      <c r="C109" s="5" t="inlineStr">
+        <is>
+          <t>Browse by region</t>
+        </is>
+      </c>
+      <c r="D109" s="5" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="E109" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F109" s="5" t="inlineStr">
+        <is>
+          <t>"See where green employers are hiring" (region map) fourth</t>
+        </is>
+      </c>
+      <c r="G109" s="5" t="inlineStr"/>
+      <c r="H109" s="5" t="inlineStr"/>
+    </row>
+    <row r="110">
+      <c r="A110" s="5" t="inlineStr">
+        <is>
+          <t>R109</t>
+        </is>
+      </c>
+      <c r="B110" s="5" t="inlineStr">
+        <is>
+          <t>UK: homepage order</t>
+        </is>
+      </c>
+      <c r="C110" s="5" t="inlineStr">
+        <is>
+          <t>Salary insights</t>
+        </is>
+      </c>
+      <c r="D110" s="5" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="E110" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F110" s="5" t="inlineStr">
+        <is>
+          <t>"Salary insight" fifth</t>
+        </is>
+      </c>
+      <c r="G110" s="5" t="inlineStr"/>
+      <c r="H110" s="5" t="inlineStr"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="5" t="inlineStr">
+        <is>
+          <t>R110</t>
+        </is>
+      </c>
+      <c r="B111" s="5" t="inlineStr">
+        <is>
+          <t>UK: homepage order</t>
+        </is>
+      </c>
+      <c r="C111" s="5" t="inlineStr">
+        <is>
+          <t>Why GreenJobs</t>
+        </is>
+      </c>
+      <c r="D111" s="5" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="E111" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F111" s="5" t="inlineStr">
+        <is>
+          <t>"Why GreenJobs" sixth</t>
+        </is>
+      </c>
+      <c r="G111" s="5" t="inlineStr"/>
+      <c r="H111" s="5" t="inlineStr"/>
+    </row>
+    <row r="112">
+      <c r="A112" s="5" t="inlineStr">
+        <is>
+          <t>R111</t>
+        </is>
+      </c>
+      <c r="B112" s="5" t="inlineStr">
+        <is>
+          <t>UK: homepage order</t>
+        </is>
+      </c>
+      <c r="C112" s="5" t="inlineStr">
+        <is>
+          <t>Employers and advertising</t>
+        </is>
+      </c>
+      <c r="D112" s="5" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="E112" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F112" s="5" t="inlineStr">
+        <is>
+          <t>"Employers and advertising" seventh</t>
+        </is>
+      </c>
+      <c r="G112" s="5" t="inlineStr"/>
+      <c r="H112" s="5" t="inlineStr"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="5" t="inlineStr">
+        <is>
+          <t>R112</t>
+        </is>
+      </c>
+      <c r="B113" s="5" t="inlineStr">
+        <is>
+          <t>UK: homepage order</t>
+        </is>
+      </c>
+      <c r="C113" s="5" t="inlineStr">
+        <is>
+          <t>Job alerts</t>
+        </is>
+      </c>
+      <c r="D113" s="5" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="E113" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F113" s="5" t="inlineStr">
+        <is>
+          <t>"Job alerts: the week's green roles, in your inbox" last</t>
+        </is>
+      </c>
+      <c r="G113" s="5" t="inlineStr"/>
+      <c r="H113" s="5" t="inlineStr"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="5" t="inlineStr">
+        <is>
+          <t>R113</t>
+        </is>
+      </c>
+      <c r="B114" s="5" t="inlineStr">
+        <is>
+          <t>UK: homepage order</t>
+        </is>
+      </c>
+      <c r="C114" s="5" t="inlineStr">
+        <is>
+          <t>The animated “Map, Pay, Sectors” sequence could be reduced to one compact insights section.</t>
+        </is>
+      </c>
+      <c r="D114" s="5" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="E114" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F114" s="5" t="inlineStr">
+        <is>
+          <t>No animated Map/Pay/Sectors sequence; static region map + salary tiles</t>
+        </is>
+      </c>
+      <c r="G114" s="5" t="inlineStr"/>
+      <c r="H114" s="5" t="inlineStr"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="5" t="inlineStr">
+        <is>
+          <t>R114</t>
+        </is>
+      </c>
+      <c r="B115" s="5" t="inlineStr">
+        <is>
+          <t>UK: network positioning</t>
+        </is>
+      </c>
+      <c r="C115" s="5" t="inlineStr">
+        <is>
+          <t>Make the network much more prominent: Advertise once. Reach candidates across the GreenJobs specialist network. Your vacancy is automatically distributed to the most relevant environmental, ecology, renewable-energy, water, waste, wind and solar job sites.</t>
+        </is>
+      </c>
+      <c r="D115" s="5" t="inlineStr">
+        <is>
+          <t>IE+UK</t>
+        </is>
+      </c>
+      <c r="E115" s="5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F115" s="5" t="inlineStr">
+        <is>
+          <t>Exact text as h1 + lede on /uk/employers/ and /ie/employers/, and as the home employer section lede</t>
+        </is>
+      </c>
+      <c r="G115" s="5" t="inlineStr"/>
+      <c r="H115" s="5" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:H115"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -837,7 +5002,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2470,7 +6635,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3819,7 +7984,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4270,7 +8435,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
[greenjobs] Human-eye rounds 3–4: sticky package-table header below 1200px only, salary Min/Max labels with €/£ prefix, job-description label + help, dashboard one-sentence tiles (no clamp), separator pairs shared Py/JS (sep_pair/sepPair), single Location row and matching hero chip, dark segmented control, treemap wrap/short-name labels, NI muted in dark map, county counts at 390, one salary band set on every device, subscribe note, fit-card serif titles, 404 wordmark, employers note merge; CSS line-joining in publish_text; sepPair + css publish tests; layout baselines refreshed; human-eye verdict + round logs; checklist E4 and COVERAGE.md corrected; test register refreshed (3,047 checks)
Co-Authored-By: Claude <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XyZXNeMjVmnqRyKctLtDmB
</commit_message>
<xml_diff>
--- a/deliverables/greenjobs_redesign_2026-09-22/tests_register_2026-09-28.xlsx
+++ b/deliverables/greenjobs_redesign_2026-09-22/tests_register_2026-09-28.xlsx
@@ -15,6 +15,7 @@
     <sheet name="Not automatable" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Automated Python" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Automated Node" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Human-eye rounds" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Keith requirements'!$A$1:$H$115</definedName>
@@ -492,7 +493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -513,6 +514,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
@@ -521,7 +523,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>PASS — 165 roles, 195 pages, CSS 69.7/80 KB, JS 97.8/125 KB</t>
+          <t>PASS — 165 roles, 195 pages, CSS 79.3/80 KB, JS 111.3/125 KB (2026-09-30)</t>
         </is>
       </c>
     </row>
@@ -533,7 +535,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>84 test functions; 1,010 checks; 0 failed, 0 skipped</t>
+          <t>1,258 checks (build + validate + scrape + gaps); 0 failed, 0 skipped (2026-09-30)</t>
         </is>
       </c>
     </row>
@@ -545,7 +547,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>40 node tests + 15 dashboard DOM checks + 1,732 layout-regression assertions (202 page loads, 3 viewports × 2 themes)</t>
+          <t>42 node tests + 15 dashboard DOM checks + 1,732 layout-regression assertions (202 page loads, 3 viewports × 2 themes); run_all.py total 3,047</t>
         </is>
       </c>
     </row>
@@ -557,7 +559,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>45 cases listed; QA lens ran 34, 28 PASS, 2 FAIL (both fixed since), 4 PARTIAL</t>
+          <t>Functional walk (walk.js) 134/134 on both editions at 1440 and 390; 45 manual cases listed</t>
         </is>
       </c>
     </row>
@@ -642,6 +644,56 @@
       <c r="B14" t="inlineStr">
         <is>
           <t>research/qa_2026-09-28/: requirements matrix v1+v2, visual sweeps v1+v2, acceptance walk v3, panel re-run findings, pipeline audit v2</t>
+        </is>
+      </c>
+    </row>
+    <row r="15"/>
+    <row r="16"/>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Human-eye release gate (skill human-eye-test)</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>4 rounds, 180-shot matrix read image by image; r1 37 → r2 20 → r3 13 → r4 8 defects; all P1/P2 fixed, 3 P3 accepted; verdict: research/qa_2026-09-28/human_eye_verdict.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Site-manager requests (2026-09-29)</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Package table Premium posting + Membership only; full job-description preview — both editions, verified by walk.js B1–B4 and pipeline audit</t>
         </is>
       </c>
     </row>
@@ -7047,7 +7099,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E85"/>
+  <dimension ref="A1:E86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -8718,6 +8770,26 @@
       </c>
       <c r="E85" s="4" t="n">
         <v>383</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="n">
+        <v>85</v>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>test_publish_text</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>publish_text(css=True) joins after { } ; , only; quoted ; kept</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -8732,7 +8804,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B41"/>
+  <dimension ref="A1:B42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -9231,8 +9303,202 @@
         </is>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>lib.test.js</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:B41"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="90" customWidth="1" min="6" max="6"/>
+    <col width="55" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Round</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Defects found</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Accepted</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Highlights</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Evidence file</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>r1</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>37</v>
+      </c>
+      <c r="D2" t="n">
+        <v>37</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>mobile table Standard column, map chips, cross-page stats mismatch, closed/unverified job headers</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>research/qa_2026-09-28/human_eye/DEFECTS.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>r2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>20</v>
+      </c>
+      <c r="D3" t="n">
+        <v>20</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>separator pairs, dark carousel mask, Membership ticks, sterling source line, NI map label</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>research/qa_2026-09-28/human_eye/DEFECTS_r2.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>r3</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>13</v>
+      </c>
+      <c r="D4" t="n">
+        <v>13</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>sticky thead at 1024, salary labels + €/£ prefix, dashboard tile copy, single Location row, treemap labels</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>research/qa_2026-09-28/human_eye/DEFECTS_r3.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>r4</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>8</v>
+      </c>
+      <c r="D5" t="n">
+        <v>5</v>
+      </c>
+      <c r="E5" t="n">
+        <v>3</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>dashboard clamp removed, one salary band set on every device, UK/IE chip wording, subscribe copy; accepted: 1024 chart label size, cookie dialog focus, wrapped snapshot chip</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>research/qa_2026-09-28/human_eye_verdict.md</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>